<commit_message>
Log initial National Proficiency app concept
Capture the client's first description of the app (launch animation,
login, profile page, Home tab, messaging tab) as scope items (S-001
to S-005), open questions (Q-001 to Q-007), and capability map rows
(CAP-001 to CAP-005). Sync all companion Markdown files and log 4
confirmed decisions. Proposal readiness remains NOT READY pending 4
P0 questions (business domain, rank system, medal system, account/
auth rules).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -195,7 +195,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Column A = labels, Column B = details. All values currently marked TBD — this tab updates automatically in wording as real project information comes in. Nothing here is a guess; anything not yet confirmed is left as TBD.</t>
+        <t>Column A = labels, Column B = details. Anything not yet confirmed by the client is left as TBD or flagged with the related Q-### question -- nothing here is guessed.</t>
       </text>
     </comment>
   </commentList>
@@ -210,7 +210,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>ID prefixes: S-### scope items, Q-### open questions, R-### risks, F-### future ideas. Priority: P0 proposal blocker, P1 first version, P2 can wait, P3 future/optional. Row 2 is an EXAMPLE (italic gray) — delete it once real rows are added; do not delete the header row.</t>
+        <t>ID prefixes: S-### scope items, Q-### open questions, R-### risks, F-### future ideas. Priority: P0 proposal blocker, P1 first version, P2 can wait, P3 future/optional.</t>
       </text>
     </comment>
   </commentList>
@@ -225,7 +225,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>IDs use QA-### internally; describe this tab to the client as “review-ready items.” Row 2 is an EXAMPLE (italic gray) — delete it once real rows are added.</t>
+        <t>IDs use QA-### internally; describe this tab to the client as review-ready items. No items are clear enough for review yet -- row 2 stays an EXAMPLE (italic gray) until a real item qualifies.</t>
       </text>
     </comment>
   </commentList>
@@ -240,7 +240,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Cypress Coverage / Command values: Not built yet / Manual review only / Future automation target / Needs technical review. Cypress Closure Status values: Open / Not Started / Needs Clarification / Confirmed / Future Phase / Ready for Review. Row 2 is an EXAMPLE (italic gray) — delete once real rows are added.</t>
+        <t>Cypress Coverage / Command values: Not built yet / Manual review only / Future automation target / Needs technical review. Cypress Closure Status values: Open / Not Started / Needs Clarification / Confirmed / Future Phase / Ready for Review.</t>
       </text>
     </comment>
   </commentList>
@@ -255,7 +255,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Dump raw/messy input here first (meeting notes, screenshots described in text, client messages, brainstorming). Anything unclear should be promoted into Scope Items as a Q-### row. Row 2 is an EXAMPLE (italic gray) — delete once real rows are added.</t>
+        <t>Dump raw/messy input here first (meeting notes, screenshots described in text, client messages, brainstorming). Anything unclear should be promoted into Scope Items as a Q-### row.</t>
       </text>
     </comment>
   </commentList>
@@ -555,7 +555,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -570,7 +570,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Project Name</t>
@@ -582,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Updated</t>
@@ -594,7 +594,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Current Understanding</t>
@@ -602,11 +602,11 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>TBD — awaiting initial project information from client/stakeholders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+          <t>National Proficiency is a native mobile app (iOS + Android). Confirmed flow: branded launch animation -&gt; username/password login -&gt; individual profile page (user photo, current rank, medals/achievements earned, guidance on the next accomplishment) -&gt; Home tab (updates, monthly challenges, a community aspect) -&gt; a second tab, next to Home, for messaging/community communication. What proficiency the app actually tracks (e.g. fitness, professional certification, military/first-responder training, other) has not been stated yet -- see Q-001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Business Goal</t>
@@ -614,11 +614,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TBD — awaiting confirmation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>TBD -- not yet stated by the client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Highest Priority Next</t>
@@ -626,11 +626,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>TBD — no scope items captured yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>Resolve P0 open questions blocking the core screens: business domain/goal (Q-001), the rank and medal/achievement system (Q-002, Q-003), and account provisioning/authentication rules (Q-005).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Verification Required</t>
@@ -638,11 +638,11 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>TBD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>Client confirmation of the full navigation structure, rank/medal rules, monthly-challenge mechanics, and whether the Home tab's 'community aspect' is the same feature as the separate Messaging tab or a distinct one (Q-004).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Open Decisions</t>
@@ -650,11 +650,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>TBD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>Login mechanism (username/password, not SSO), profile page as the post-login landing screen, and tab order (Home, then Messaging second) -- see DECISIONS.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Proposal Notes</t>
@@ -662,7 +662,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Worksheet structure created. No scope content entered yet — not ready for proposal.</t>
+          <t>Initial app concept received: 5 workflows (onboarding animation, login, profile, home, messaging). Still not proposal-ready -- multiple P0 items open. See PROPOSAL_READINESS.md.</t>
         </is>
       </c>
     </row>
@@ -678,20 +678,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -751,56 +751,639 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>S-001 (EXAMPLE)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Initial Discovery</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Q-001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Admin dashboard</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Role-based access for program administrators</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Database / records</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>What is National Proficiency's core business/domain -- what proficiency is being tracked (fitness, martial arts, professional certification, military/first-responder training, other)?</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Full business description and objective for the app.</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Database / records</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation in writing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Q-002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>What are the specific ranks/levels in the progression system, and what are the criteria to advance from one to the next?</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Full rank list and advancement rules per rank.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided rank list; QA against one test account per rank tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Q-003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>What are the specific medals/achievements available, and how is each one earned?</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Full medal/achievement list and the criteria to earn each.</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided medal list and earn criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Q-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Is the Home tab's 'community aspect' the same feature as the separate messaging/community tab, or two distinct features? If distinct, what belongs on Home vs. in Messaging?</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Client clarification separating Home content from Messaging tab content.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Notifications</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; wireframe review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Q-005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>How are accounts created -- self-registration, admin/organization-issued, or invite-only? Is a password-reset flow required? Is MFA required?</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Account provisioning model, password-reset requirement, MFA requirement.</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>User management / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; acceptance criteria for login states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Q-006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>How are monthly challenges created, tracked, and scored? Are there prizes or recognition tied to completion?</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Challenge creation process, tracking/scoring rules, and any reward mechanics.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided example of one full monthly challenge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Q-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>What is the full tab-bar/navigation structure beyond the profile page (post-login landing) and Home + Messaging? Are there additional tabs (e.g. Settings, Notifications)?</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Complete list and order of app tabs/navigation.</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided navigation map or wireframe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>S-001</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Public form / Onboarding</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Branded app launch animation ("National Proficiency") shown on open, before login.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Confirm animation length/style, brand assets (logo, colors, motion), whether it's skippable, and behavior on slow network/cold start.</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Public form / Onboarding (mobile splash screen)</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Client sign-off on animation mockup/video; QA of cold-start timing on iOS and Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>S-002</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Username/password login required to access an individual account.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Needs Clarification</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Confirm which roles exist and what each role can see/edit before this can be scoped.</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Admin dashboard / User management</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>Client confirmation of role list + permissions matrix</t>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Account provisioning method, password-reset flow, session/token expiration, MFA, error/lockout handling -- see Q-005.</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>User management / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Acceptance criteria for login success/failure states; client confirmation of provisioning method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>S-003</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Individual profile page: user photo, current rank, medals/achievements earned, guidance on the next accomplishment to pursue.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Full rank system, full medal/achievement list, logic/content for "what's next," and photo source (user-uploaded vs. admin-assigned) -- see Q-002, Q-003.</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of rank/medal list and progression rules; QA against a test account per rank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>S-004</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Home tab: updates feed, monthly challenges, a community aspect.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Source/authorship of updates (admin-posted vs. system-generated), monthly-challenge structure and progress tracking, and how "community aspect" differs from the Messaging tab -- see Q-004, Q-006.</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Notifications</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of content types and one example monthly challenge; QA of feed rendering per role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>S-005</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Messaging / community communications tab, positioned second, next to Home -- lets members keep each other updated.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Whether this is 1:1 direct messaging, group/team chat, or a public feed; moderation rules; push notifications; media/attachment support -- see Q-004.</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Notifications</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of message format and one example use case; QA send/receive across two test accounts.</t>
         </is>
       </c>
     </row>
@@ -969,18 +1552,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1036,55 +1619,243 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>CAP-001 (EXAMPLE)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Public form</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Prospective client submits an intake request</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Public / anonymous user</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Marketing site → “Get Started” → intake form</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>CAP-001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Public form / Onboarding</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>App launch -&gt; branded animation</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>All users (pre-login)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Open the app on iOS or Android</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Not built yet</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Confirm required fields and validation rules with client</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>QA-001</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Example: No app exists yet — plain-English area only</t>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Confirm animation assets and timing once designed.</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CAP-002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Username/password login</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Registered members</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>App launch -&gt; login screen</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Confirm account provisioning and password-reset flow (Q-005).</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-002.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CAP-003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Individual profile page (photo, rank, medals, next steps)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Logged-in member (own profile)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Login -&gt; lands on profile page</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Confirm rank and medal system (Q-002, Q-003).</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-003. Landing page immediately after login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CAP-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Home tab (updates, monthly challenges, community)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Logged-in member</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Tab bar -&gt; Home</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Confirm content sources and monthly-challenge structure (Q-004, Q-006).</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-004.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CAP-005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Messaging / community communications</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Logged-in member</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Tab bar -&gt; second tab, next to Home</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Confirm messaging model -- direct message vs. group vs. feed (Q-004).</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-005.</t>
         </is>
       </c>
     </row>
@@ -1105,9 +1876,9 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1137,30 +1908,30 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Kickoff email</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Client mentioned wanting a client portal but gave no detail on login/roles.</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Client portal</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Example: Turned into Q-001 in Scope Items — needs follow-up.</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Client described the app concept end to end: on open (Android or Apple), the app shows a branded "National Proficiency" animation, then a username/password login. After login it opens to the user's individual page with their photo on top, current rank, any medals achieved, and info on where to go next to achieve their next accomplishment. Selecting the Home page shows updates, monthly challenges, and possibly a community aspect. A second tab, next to Home, is a messaging/community-style communications section where people can keep each other updated on information or activities.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>App overview -- Onboarding / Login / Profile / Home / Messaging</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Broken into S-001 through S-005 (scope items) and Q-001 through Q-007 (open questions). Awaiting rank/medal system, account provisioning, monthly-challenge mechanics, and Home-vs-Messaging community clarification.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Media tab and membership tier structure
Capture the client's addition of a Premium-only Media tab (medical,
fitness, firearms & building training videos), account-required
access, and the Free/Mid/Premium tier structure. Add S-006, S-007
scope items; Q-008 to Q-013 open questions; R-001, R-002 risks
(raffle sweepstakes exposure, content liability); CAP-006 capability
row. Sync all companion Markdown files. Proposal readiness remains
NOT READY pending 6 P0 questions and the raffle legal risk.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="80" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Project Name</t>
@@ -582,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="80" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Updated</t>
@@ -594,7 +594,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Current Understanding</t>
@@ -602,11 +602,11 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android). Confirmed flow: branded launch animation -&gt; username/password login -&gt; individual profile page (user photo, current rank, medals/achievements earned, guidance on the next accomplishment) -&gt; Home tab (updates, monthly challenges, a community aspect) -&gt; a second tab, next to Home, for messaging/community communication. What proficiency the app actually tracks (e.g. fitness, professional certification, military/first-responder training, other) has not been stated yet -- see Q-001.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access). Confirmed flow: branded launch animation -&gt; account login -&gt; individual profile page (photo, current rank, medals/achievements, next-accomplishment guidance) -&gt; tab bar with Home (updates, monthly challenges, community aspect), Chat/Messaging, and a Media tab (medical training videos, fitness training videos, and firearms &amp; building training videos -- exact meaning of "building" videos not yet confirmed, see Q-008). Three membership tiers gate access: Free (app + profile + Home only), Mid (feature set still being defined by the client), and Premium (all features, including chats, media, challenges, monthly raffles, and additional personalized guidance). What proficiency the app tracks and its target audience is still not explicitly confirmed -- the medical/fitness/firearms content categories are a strong hint but not a confirmed answer, see Q-001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Business Goal</t>
@@ -614,11 +614,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TBD -- not yet stated by the client.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
+          <t>TBD -- not yet explicitly stated by the client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Highest Priority Next</t>
@@ -626,11 +626,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Resolve P0 open questions blocking the core screens: business domain/goal (Q-001), the rank and medal/achievement system (Q-002, Q-003), and account provisioning/authentication rules (Q-005).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+          <t>Resolve P0 items: business domain/audience (Q-001), rank system (Q-002), medal system (Q-003), account/auth rules (Q-005), mid-tier feature list and tier pricing (Q-009, Q-010), and the raffle legal/compliance risk (R-001).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Verification Required</t>
@@ -638,11 +638,11 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full navigation structure, rank/medal rules, monthly-challenge mechanics, and whether the Home tab's 'community aspect' is the same feature as the separate Messaging tab or a distinct one (Q-004).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+          <t>Client confirmation of navigation structure, rank/medal rules, monthly-challenge mechanics, Home-vs-Messaging community overlap and whether challenges are tier-gated (Q-004, Q-011), exact Media tab video categories (Q-008), and what 'additional guidance' means in practice (Q-013).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Open Decisions</t>
@@ -650,11 +650,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Login mechanism (username/password, not SSO), profile page as the post-login landing screen, and tab order (Home, then Messaging second) -- see DECISIONS.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+          <t>Login mechanism, profile-page landing screen, tab order, account-required access, and the three-tier structure and its Free/Premium boundaries are decided in direction -- see DECISIONS.md. Mid tier and all pricing remain undecided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Proposal Notes</t>
@@ -662,7 +662,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Initial app concept received: 5 workflows (onboarding animation, login, profile, home, messaging). Still not proposal-ready -- multiple P0 items open. See PROPOSAL_READINESS.md.</t>
+          <t>App concept and tier/paywall structure now captured. Still not proposal-ready -- multiple P0 items open, plus one legal/compliance risk (R-001) around the premium raffle that should be reviewed before proposing pricing or timelines. See PROPOSAL_READINESS.md.</t>
         </is>
       </c>
     </row>
@@ -678,20 +678,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -751,7 +751,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="70" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Q-001</t>
@@ -774,7 +774,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>What is National Proficiency's core business/domain -- what proficiency is being tracked (fitness, martial arts, professional certification, military/first-responder training, other)?</t>
+          <t>What is National Proficiency's core business/domain and target audience -- what proficiency is being tracked (fitness, martial arts, professional certification, military/first-responder training, other)?</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -790,7 +790,7 @@
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Full business description and objective for the app.</t>
+          <t>Full business description, target audience, and objective for the app. Partial signal: Media tab content (medical, fitness, firearms/building training) suggests a tactical/safety/professional training domain, but this has not been explicitly confirmed -- please confirm the audience and whether this is related to any existing training business on file.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="70" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Q-002</t>
@@ -857,7 +857,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Q-003</t>
@@ -910,7 +910,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="70" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Q-004</t>
@@ -963,7 +963,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="70" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Q-005</t>
@@ -1016,7 +1016,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="70" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Q-006</t>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="70" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Q-007</t>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>What is the full tab-bar/navigation structure beyond the profile page (post-login landing) and Home + Messaging? Are there additional tabs (e.g. Settings, Notifications)?</t>
+          <t>What is the full tab-bar/navigation structure? Confirmed so far: profile (post-login landing), Home, Chat/Messaging, Media. Any additional tabs (e.g. Settings, Notifications)?</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1122,10 +1122,10 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="70" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>S-001</t>
+          <t>Q-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1140,17 +1140,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Public form / Onboarding</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Branded app launch animation ("National Proficiency") shown on open, before login.</t>
+          <t>What exactly are the 'firearms and building' videos on the Media tab? Two categories (firearms training + building/facility training) or one? Please confirm the exact wording/meaning -- this may also affect legal/compliance requirements for hosting the content.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1161,24 +1161,24 @@
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Confirm animation length/style, brand assets (logo, colors, motion), whether it's skippable, and behavior on slow network/cold start.</t>
+          <t>Exact video category list and any hosting/compliance constraints per category.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Public form / Onboarding (mobile splash screen)</t>
+          <t>Client portal (Media) / Security / compliance</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Client sign-off on animation mockup/video; QA of cold-start timing on iOS and Android.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
+          <t>Client confirmation of category list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>S-002</t>
+          <t>Q-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1193,17 +1193,17 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Username/password login required to access an individual account.</t>
+          <t>What features belong to the Mid membership tier? Client indicated it is still being worked out.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1214,24 +1214,24 @@
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Account provisioning method, password-reset flow, session/token expiration, MFA, error/lockout handling -- see Q-005.</t>
+          <t>Final Mid-tier feature list -- needed before tier-gating logic can be designed or built.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>User management / Security / compliance</t>
+          <t>Payments / User management</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Acceptance criteria for login success/failure states; client confirmation of provisioning method.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+          <t>Client-provided tier feature matrix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>S-003</t>
+          <t>Q-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Individual profile page: user photo, current rank, medals/achievements earned, guidance on the next accomplishment to pursue.</t>
+          <t>What is the price of each membership tier (Free/Mid/Premium), and what payment processor/billing system should be used (subscriptions, trials, upgrade/downgrade handling)?</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1267,24 +1267,24 @@
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Full rank system, full medal/achievement list, logic/content for "what's next," and photo source (user-uploaded vs. admin-assigned) -- see Q-002, Q-003.</t>
+          <t>Pricing per tier and billing platform decision -- needed to scope the Payments build area and for the proposal itself.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of rank/medal list and progression rules; QA against a test account per rank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+          <t>Client-provided pricing; confirmation of payment processor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>S-004</t>
+          <t>Q-011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Home tab: updates feed, monthly challenges, a community aspect.</t>
+          <t>Monthly challenges are described as part of the Home tab (S-004), but the Free tier is described as not having access to challenges. Does that mean challenges appear on Home but are gated per-tier, or are challenges a separate screen outside Home? Also: is the Home 'community aspect' gated by tier, or available to all logged-in users including Free?</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1320,24 +1320,24 @@
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Source/authorship of updates (admin-posted vs. system-generated), monthly-challenge structure and progress tracking, and how "community aspect" differs from the Messaging tab -- see Q-004, Q-006.</t>
+          <t>Clarify how tier-gating applies within the Home tab specifically.</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>Client portal / Payments</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of content types and one example monthly challenge; QA of feed rendering per role.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+          <t>Client confirmation; wireframe review of Home tab per tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>S-005</t>
+          <t>Q-012</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1352,17 +1352,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Messaging / community communications tab, positioned second, next to Home -- lets members keep each other updated.</t>
+          <t>How does the Premium-tier 'monthly raffle for challenges' work -- how are winners selected, what are the prizes, and who administers it?</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1373,17 +1373,547 @@
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Whether this is 1:1 direct messaging, group/team chat, or a public feed; moderation rules; push notifications; media/attachment support -- see Q-004.</t>
+          <t>Raffle mechanics and administration process. See related risk R-001 on legal/compliance exposure.</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
+          <t>Payments / AI workflow</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided raffle rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Q-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>What does 'additional guidance based on things they're working on' (a Premium-tier perk) mean concretely -- human coach/trainer feedback, AI-generated recommendations, or something else, and how is it delivered in-app?</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Definition of the guidance feature, who/what produces it, and delivery mechanism (in-app messages, notifications, reports, etc.).</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / AI workflow</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; one worked example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>R-001</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Premium tier includes a monthly raffle tied to challenges. Paying for a subscription that includes a chance to win something can implicate sweepstakes/lottery/gambling law depending on jurisdiction.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Legal/compliance review of the raffle mechanic before it is built or promoted -- may require an alternate no-purchase-necessary entry path or a redesign of the reward mechanic.</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / Payments</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Sign-off from client's legal counsel or compliance advisor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>R-002</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>The Media tab hosts firearms training and medical training video content, which may carry liability, age-verification, or regulatory considerations depending on jurisdiction and audience.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Legal/compliance review of content liability and any age/identity verification needed before granting Media tab access.</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Sign-off from client's legal counsel or compliance advisor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>S-001</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Public form / Onboarding</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Branded app launch animation ("National Proficiency") shown on open, before login.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Confirm animation length/style, brand assets (logo, colors, motion), whether it's skippable, and behavior on slow network/cold start.</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Public form / Onboarding (mobile splash screen)</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Client sign-off on animation mockup/video; QA of cold-start timing on iOS and Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>S-002</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Account required for all app access -- no guest/anonymous use. New users create an account and select a membership tier; existing users log in with username/password.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Account provisioning method, password-reset flow, session/token expiration, MFA, error/lockout handling (Q-005); confirm tier selection happens at sign-up (see S-007).</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>User management / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Acceptance criteria for login success/failure states; client confirmation of provisioning method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>S-003</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Individual profile page: user photo, current rank, medals/achievements earned, guidance on the next accomplishment to pursue.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Full rank system, full medal/achievement list, logic/content for "what's next," and photo source (user-uploaded vs. admin-assigned) -- see Q-002, Q-003.</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of rank/medal list and progression rules; QA against a test account per rank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>S-004</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Home tab: updates feed, monthly challenges, a community aspect. Free tier is described as excluding challenges.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Source/authorship of updates, monthly-challenge structure and progress tracking (Q-006), how 'community aspect' differs from the Messaging tab (Q-004), and how tier-gating applies within this single tab (Q-011).</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
           <t>Client portal / Notifications</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>Client confirmation of message format and one example use case; QA send/receive across two test accounts.</t>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of content types and one example monthly challenge; QA of feed rendering per role and per tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>S-005</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Messaging / community communications tab, positioned second next to Home. Free tier is described as excluding chats; Premium tier includes them.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Whether this is 1:1 direct messaging, group/team chat, or a public feed; moderation rules; push notifications; media/attachment support (Q-004); confirm Mid-tier access level once defined (Q-009).</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Notifications</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of message format and one example use case; QA send/receive across two test accounts per eligible tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>S-006</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media)</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Media hosting tab (after Home and Chat), accessible only to premium subscribers: hosts medical training videos, fitness training videos, and firearms &amp; building training videos.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Exact video category definitions (Q-008), video hosting/CDN/storage approach, who uploads content (admin only, presumably), streaming vs. download, captioning/accessibility, and any content liability/compliance review (R-002).</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media) / Database / records</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided sample video and category list; QA of playback and tier-gating (Premium-only access denied to Free/Mid test accounts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="70" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>S-007</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Three membership tiers gate feature access. Free: app, profile page, Home page only -- no chats, media, or monthly challenges. Mid: feature set still being defined by the client. Premium: all features, plus monthly raffles tied to challenges, media access, chats, and additional personalized guidance.</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Full Mid-tier feature list (Q-009), pricing per tier and billing platform (Q-010), upgrade/downgrade flow, and legal review of the raffle mechanic (R-001). This gates the build of nearly every other feature via entitlement/paywall logic.</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Payments / User management</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided tier feature matrix and pricing; QA of access boundaries per tier using one test account per tier.</t>
         </is>
       </c>
     </row>
@@ -1552,19 +2082,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1619,7 +2149,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>CAP-001</t>
@@ -1667,7 +2197,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="55" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>CAP-002</t>
@@ -1680,17 +2210,17 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Username/password login</t>
+          <t>Account creation / login (account required for all access)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Registered members</t>
+          <t>New and returning users</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>App launch -&gt; login screen</t>
+          <t>App launch -&gt; login/sign-up screen</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -1705,17 +2235,17 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Confirm account provisioning and password-reset flow (Q-005).</t>
+          <t>Confirm account provisioning, password-reset flow, and tier selection at sign-up (Q-005, S-007).</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Relates to S-002.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="45" customHeight="1">
+          <t>Relates to S-002, S-007.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>CAP-003</t>
@@ -1733,7 +2263,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Logged-in member (own profile)</t>
+          <t>Logged-in member (own profile), all tiers</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1763,7 +2293,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>CAP-004</t>
@@ -1781,7 +2311,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Logged-in member</t>
+          <t>Logged-in member, all tiers (challenges may be Premium/Mid only)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1801,7 +2331,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Confirm content sources and monthly-challenge structure (Q-004, Q-006).</t>
+          <t>Confirm content sources, challenge structure, and per-tier gating within Home (Q-004, Q-006, Q-011).</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
@@ -1811,7 +2341,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>CAP-005</t>
@@ -1829,12 +2359,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Logged-in member</t>
+          <t>Premium tier confirmed; Free tier excluded; Mid tier TBD</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Tab bar -&gt; second tab, next to Home</t>
+          <t>Tab bar -&gt; Chat tab, next to Home</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1849,13 +2379,61 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Confirm messaging model -- direct message vs. group vs. feed (Q-004).</t>
+          <t>Confirm messaging model (Q-004) and Mid-tier access (Q-009).</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Relates to S-005.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CAP-006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Media hosting -- medical, fitness, and firearms/building training videos</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Premium tier only; Free and Mid excluded (Mid TBD)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Tab bar -&gt; Media tab</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Confirm video categories (Q-008), hosting approach, and content liability review (R-002).</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-006. New tab added after Home and Chat.</t>
         </is>
       </c>
     </row>
@@ -1871,14 +2449,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1908,7 +2486,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="100" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1932,6 +2510,33 @@
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Broken into S-001 through S-005 (scope items) and Q-001 through Q-007 (open questions). Awaiting rank/medal system, account provisioning, monthly-challenge mechanics, and Home-vs-Messaging community clarification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Client added: a Media tab after Home/Chat/Profile, premium-subscribers only, hosting medical training videos, fitness training videos, and firearms &amp; building training videos (exact meaning of "building" unconfirmed). Whole app requires an account -- no guest access; new users create an account. Three tiers: Free (app + profile + Home, no chats/media/challenges), Mid ("being worked on" -- not yet defined by client), Premium (all features + monthly raffles tied to challenges + media + chats + additional personalized guidance based on what the user is working on).</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>App overview -- Media tab / Membership tiers / Paywall</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Broken into S-006, S-007 (scope items), Q-008 through Q-013 (open questions), and R-001, R-002 (risks). Flagged: challenges were placed on Home (S-004) but Free tier excludes challenges -- gating logic within Home needs clarification (Q-011). Flagged: raffle tied to paid tier may have legal/compliance exposure (R-001).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm National Proficiency is separate from Tactical Rabbi
Client confirmed National Proficiency and Tactical Rabbi are
completely unrelated brands with no information crossover. Closes
the Tactical Rabbi sub-question inside Q-001; core business
description/audience question remains open.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access). Confirmed flow: branded launch animation -&gt; account login -&gt; individual profile page (photo, current rank, medals/achievements, next-accomplishment guidance) -&gt; tab bar with Home (updates, monthly challenges, community aspect), Chat/Messaging, and a Media tab (medical training videos, fitness training videos, and firearms &amp; building training videos -- exact meaning of "building" videos not yet confirmed, see Q-008). Three membership tiers gate access: Free (app + profile + Home only), Mid (feature set still being defined by the client), and Premium (all features, including chats, media, challenges, monthly raffles, and additional personalized guidance). What proficiency the app tracks and its target audience is still not explicitly confirmed -- the medical/fitness/firearms content categories are a strong hint but not a confirmed answer, see Q-001.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access). Confirmed flow: branded launch animation -&gt; account login -&gt; individual profile page (photo, current rank, medals/achievements, next-accomplishment guidance) -&gt; tab bar with Home (updates, monthly challenges, community aspect), Chat/Messaging, and a Media tab (medical training videos, fitness training videos, and firearms &amp; building training videos -- exact meaning of "building" videos not yet confirmed, see Q-008). Three membership tiers gate access: Free (app + profile + Home only), Mid (feature set still being defined by the client), and Premium (all features, including chats, media, challenges, monthly raffles, and additional personalized guidance). National Proficiency is confirmed to be a completely separate brand/company from Tactical Rabbi, with no crossover of information between the two -- treat them as fully unrelated projects. What proficiency the app tracks and its target audience is still not explicitly confirmed, see Q-001.</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>What is National Proficiency's core business/domain and target audience -- what proficiency is being tracked (fitness, martial arts, professional certification, military/first-responder training, other)?</t>
+          <t>What is National Proficiency's core business/domain and target audience -- what proficiency is being tracked (fitness, martial arts, professional certification, military/first-responder training, other)? CONFIRMED: National Proficiency is a completely separate brand/company from Tactical Rabbi, with no crossover of information between the two -- that sub-question is closed.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -790,7 +790,7 @@
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Full business description, target audience, and objective for the app. Partial signal: Media tab content (medical, fitness, firearms/building training) suggests a tactical/safety/professional training domain, but this has not been explicitly confirmed -- please confirm the audience and whether this is related to any existing training business on file.</t>
+          <t>Full business description, target audience, and objective for the app. Media tab content (medical, fitness, firearms/building training) suggests a tactical/safety/professional training domain, but the specific business description and audience still need to be stated explicitly.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -2449,7 +2449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2540,6 +2540,33 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="100" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmed National Proficiency and Tactical Rabbi are completely separate brands/companies, not associated, with no crossover of information between the two projects.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>App overview -- Business context</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Resolved the Tactical Rabbi sub-question inside Q-001 (closed). Core Q-001 business-description/audience question remains open. Flagged a repo-hygiene question to the client: both projects currently live in the same git repository -- asked whether National Proficiency's docs should move to a separate repo to guarantee no crossover.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log instructor/backend qualification workflow
Capture the client's description of the Approved Instructor role,
student pre-registration ("+" button), Google Calendar integration,
qualification standards library, Shooter's Global shot-timer
integration, and strict pass/fail grading with a mandatory edit
audit trail. Add S-008 to S-013 scope items, Q-014 to Q-018 open
questions, R-003 risk (qualification record-keeping compliance),
and CAP-007/CAP-008 capability rows. Update Q-001 to Q-003 and S-003
to reflect the now-confirmed rank/medal earning mechanism. Sync all
companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access). Confirmed flow: branded launch animation -&gt; account login -&gt; individual profile page (photo, current rank, medals/achievements, next-accomplishment guidance) -&gt; tab bar with Home (updates, monthly challenges, community aspect), Chat/Messaging, and a Media tab (medical training videos, fitness training videos, and firearms &amp; building training videos -- exact meaning of "building" videos not yet confirmed, see Q-008). Three membership tiers gate access: Free (app + profile + Home only), Mid (feature set still being defined by the client), and Premium (all features, including chats, media, challenges, monthly raffles, and additional personalized guidance). National Proficiency is confirmed to be a completely separate brand/company from Tactical Rabbi, with no crossover of information between the two -- treat them as fully unrelated projects. What proficiency the app tracks and its target audience is still not explicitly confirmed, see Q-001.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). Confirmed user-side flow: branded launch animation -&gt; account login -&gt; individual profile page (photo, current rank, medals/achievements, next-accomplishment guidance) -&gt; tab bar with Home (updates, monthly challenges, community aspect), Chat/Messaging, and a Media tab (medical, fitness, and firearms &amp; building training videos). Three membership tiers gate access: Free (app + profile + Home only), Mid (feature set still being defined by the client), and Premium (all features, including chats, media, challenges, monthly raffles, and additional personalized guidance). The three proficiency pillars are confirmed: Medical, Firearms, and Fitness. Backend/instructor side (new): Approved Instructors share the regular user's profile and access, plus an instructor-only "+" button to pre-register a student for a qualification (category/tier/date), which sends an approval confirmation and a Google Calendar invite to the student. On qualification day, the instructor follows that tier's course-of-fire standard, records results via a shot-timer integration ("Shooter's Global") or manual entry, grades strictly pass/fail with no partial credit, and any edit to results is logged in an audit trail. A Pass automatically updates the student's profile rank/medal. The target audience/business model (who takes this program) is still not stated -- see Q-001.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Resolve P0 items: business domain/audience (Q-001), rank system (Q-002), medal system (Q-003), account/auth rules (Q-005), mid-tier feature list and tier pricing (Q-009, Q-010), and the raffle legal/compliance risk (R-001).</t>
+          <t>Resolve P0 items: business audience/model (Q-001), the actual qualification standards content per category/tier (Q-002, Q-003, S-011), account/auth rules (Q-005), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), and instructor designation process (Q-015).</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of navigation structure, rank/medal rules, monthly-challenge mechanics, Home-vs-Messaging community overlap and whether challenges are tier-gated (Q-004, Q-011), exact Media tab video categories (Q-008), and what 'additional guidance' means in practice (Q-013).</t>
+          <t>Client confirmation of navigation structure, monthly-challenge mechanics, Home-vs-Messaging community overlap and tier-gating (Q-004, Q-011), exact Media tab video categories (Q-008), the pre-registration approval workflow (Q-014), Google Calendar integration approach (Q-016), and Shooter's Global integration/partner status (Q-017).</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Login mechanism, profile-page landing screen, tab order, account-required access, and the three-tier structure and its Free/Premium boundaries are decided in direction -- see DECISIONS.md. Mid tier and all pricing remain undecided.</t>
+          <t>Login mechanism, profile-page landing screen, tab order, account-required access, the three-tier structure, the three proficiency pillars, strict pass/fail grading, and the edit-audit-trail requirement are decided in direction -- see DECISIONS.md. Mid tier, all pricing, and the full qualification standards content remain undecided.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>App concept and tier/paywall structure now captured. Still not proposal-ready -- multiple P0 items open, plus one legal/compliance risk (R-001) around the premium raffle that should be reviewed before proposing pricing or timelines. See PROPOSAL_READINESS.md.</t>
+          <t>App concept, tier/paywall structure, and instructor/qualification workflow now captured. Still not proposal-ready -- multiple P0 items open, plus legal/compliance risks (R-001 raffle, R-003 qualification record-keeping) that should be reviewed before proposing pricing or timelines. See PROPOSAL_READINESS.md.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -774,7 +774,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>What is National Proficiency's core business/domain and target audience -- what proficiency is being tracked (fitness, martial arts, professional certification, military/first-responder training, other)? CONFIRMED: National Proficiency is a completely separate brand/company from Tactical Rabbi, with no crossover of information between the two -- that sub-question is closed.</t>
+          <t>What is National Proficiency's target audience and business model? CONFIRMED: the three proficiency pillars are Medical, Firearms, and Fitness, tracked via instructor-administered pass/fail qualification testing. CONFIRMED: completely separate brand/company from Tactical Rabbi, with no crossover of information between the two.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -790,7 +790,7 @@
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Full business description, target audience, and objective for the app. Media tab content (medical, fitness, firearms/building training) suggests a tactical/safety/professional training domain, but the specific business description and audience still need to be stated explicitly.</t>
+          <t>Who takes this program (e.g. security professionals, general public, a specific organization's staff), and the business model (training academy selling courses, internal org cert tracking, other) -- still needs to be stated explicitly.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>What are the specific ranks/levels in the progression system, and what are the criteria to advance from one to the next?</t>
+          <t>What are the specific ranks/levels in the progression system, and what are the criteria to advance from one to the next? Mechanism now confirmed: ranks are earned by passing instructor-administered qualifications (S-011, S-013). Still needed: the actual rank/tier list.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -843,7 +843,7 @@
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Full rank list and advancement rules per rank.</t>
+          <t>Full rank list and advancement rules per rank -- likely best provided as the actual qualification standards documents (see S-011) rather than described verbally.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>What are the specific medals/achievements available, and how is each one earned?</t>
+          <t>What are the specific medals/achievements available, and how is each one earned? Mechanism now confirmed: a medal/badge is awarded automatically when an instructor marks a qualification Pass (S-013). Still needed: the actual medal/achievement list per category/tier.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -896,7 +896,7 @@
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Full medal/achievement list and the criteria to earn each.</t>
+          <t>Full medal/achievement list and the qualification each one maps to.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -1691,7 +1691,7 @@
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Full rank system, full medal/achievement list, logic/content for "what's next," and photo source (user-uploaded vs. admin-assigned) -- see Q-002, Q-003.</t>
+          <t>Earning mechanism now confirmed: rank/medals update automatically when an instructor marks a qualification Pass (S-013). Still needed: full rank/tier list, full medal/achievement list, logic/content for "what's next," and photo source -- see Q-002, Q-003.</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -1914,6 +1914,642 @@
       <c r="K23" s="3" t="inlineStr">
         <is>
           <t>Client-provided tier feature matrix and pricing; QA of access boundaries per tier using one test account per tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="70" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Q-014</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>When a pre-registration is submitted, does it require a separate approval step by someone else, or does "approval information" just mean an automatic confirmation is generated and sent to the student? Please clarify the approval workflow.</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Clear description of the approval step(s), if any, between submission and a confirmed registration.</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="70" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Q-015</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>How are instructors granted "Approved Instructor" status, and is certification per-category (e.g. an instructor certified for Firearms only couldn't administer Medical or Fitness qualifications)?</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Instructor approval/designation process and whether category-specific certification applies.</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Q-016</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>What does the Google Calendar integration require in practice -- the student's personal Google Calendar (needing their OAuth consent), a shared/organizational calendar, or something else? What happens if the student has no Google account?</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed calendar integration approach and no-Google-account fallback.</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="70" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Q-017</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Is "Shooter's Global" a confirmed technical/partner integration, and what interface does it expose for the app to receive shot-timer results (API, Bluetooth, file import, etc.)?</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation of partner status and technical integration details, or confirmation this is a future/aspirational integration.</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; technical documentation from Shooter's Global if a partnership exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Q-018</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Is there a retest or appeal policy after a student fails a qualification (e.g. how soon can they re-register, is there a cap on attempts)?</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Retest/appeal policy, if any.</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>R-003</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Qualification records (especially firearms and medical) likely carry legal/compliance requirements around record retention, access control, and edit chain-of-custody -- reinforced by the client's explicit request for an audit trail on edits.</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Legal/compliance review of qualification record-keeping requirements: retention period, who can access records, and whether the audit-trail format meets any applicable regulatory standard. Related to R-001, R-002.</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Sign-off from client's legal counsel or compliance advisor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="70" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>S-008</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Approved Instructor role: same profile and access to all regular-user features/pages, plus an instructor-only "+" button (center bottom of the app) that opens qualification-administration tools.</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>How instructors are designated/approved, whether certification is per-category, and how the "+" button and instructor tools stay hidden from non-instructor users -- see Q-015.</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / User management</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of instructor designation process; QA that the "+" button appears only for instructor accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="70" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>S-009</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Student pre-registration form (via the "+" button): instructor selects category (Medical / Firearms / Fitness), level/tier, and qualification date, then submits for approval.</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Full field list beyond category/tier/date (e.g. student lookup/ID, location), whether "approval" is a separate review step or an automatic confirmation, and duplicate/reschedule/cancellation handling -- see Q-014.</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / Database / records</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of full form fields and approval workflow; QA of a full registration end to end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="70" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>S-010</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Google Calendar integration: on submission, sends the qualification date to the student so they know it's recorded and scheduled.</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Whether this targets the student's personal Google Calendar or an organizational calendar, behavior with no Google account, time zone handling, and updates on reschedule/cancellation -- see Q-016.</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of calendar integration approach; QA of invite delivery and reschedule/cancel sync.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="70" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>S-011</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Qualification standards library: on the day of testing, the instructor has access to that tier's qualification standard/course of fire to follow while administering the test.</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>The actual standards/course-of-fire content for every category x tier combination (ties directly to Q-002, Q-003 -- likely needs to come from the client as source documents), format as a structured checklist, and who maintains/updates standards over time.</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / Database / records</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Client to provide the qualification standard documents for at least one category/tier as a working example; QA that the correct standard loads for the selected category/tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="70" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>S-012</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Shot timer integration ("Shooter's Global"): shot-timer drill times can be recorded directly into the app during a firearms qualification.</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Whether Shooter's Global is a confirmed technical/partner integration and what interface it exposes, what data is captured per drill, and fallback behavior if unavailable -- see Q-017.</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of integration method/partner status; QA of a recorded drill time populating correctly, and of the manual-entry fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="70" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>S-013</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Qualification grading: instructor checks off each individual qualification criterion (manual notes supported) and grades strictly pass/fail -- no partial/leniency. Any edit to recorded results is logged with an audit trail. On Pass, the student's profile automatically updates with the new medal/badge/accomplishment.</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Exact checklist criteria per category/tier (ties to S-011, Q-002, Q-003), audit-trail format (who/when/what changed, and whether it's visible to the student), retest/appeal policy after a Fail -- see Q-018. Directly updates the profile page built in S-003.</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / Database / records / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the pass/fail checklist for one example qualification; QA that an edit after submission creates a visible audit entry; QA that a Pass updates the student's profile rank/medal.</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2437,6 +3073,102 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>CAP-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Instructor pre-registration ("+" button)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Approved Instructors only</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Tab bar -&gt; center "+" button -&gt; registration form (category / tier / date) -&gt; submit</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Confirm approval workflow (Q-014), full form fields, and Google Calendar integration approach (Q-016).</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-008, S-009, S-010.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CAP-008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Qualification administration &amp; grading (course of fire, shot timer / manual entry, pass-fail checklist, audit trail)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Approved Instructors only</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Open a registered qualification on test day -&gt; standard/checklist -&gt; record results -&gt; Pass/Fail</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Confirm qualification standards content (Q-002, Q-003), Shooter's Global integration (Q-017), and retest policy (Q-018).</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-011, S-012, S-013. A Pass updates the student's profile (S-003).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -2449,7 +3181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2563,7 +3295,34 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Resolved the Tactical Rabbi sub-question inside Q-001 (closed). Core Q-001 business-description/audience question remains open. Flagged a repo-hygiene question to the client: both projects currently live in the same git repository -- asked whether National Proficiency's docs should move to a separate repo to guarantee no crossover.</t>
+          <t>Resolved the Tactical Rabbi sub-question inside Q-001 (closed). Core Q-001 business-description/audience question remains open. Flagged a repo-hygiene question to the client: both projects currently live in the same git repository -- asked whether National Proficiency's docs should move to a separate repo to guarantee no crossover. Client chose to move to a separate repo; blocked on the client creating an empty GitHub repo, since this session's GitHub integration cannot create new repositories (403 permission error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="100" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Client described the instructor/backend side: Approved Instructors share the regular user's profile and access, plus a center-bottom "+" button opening a form to pre-register a student for a qualification -- category (Medical / Firearms / Fitness), level/tier, and date. Submission produces approval information and a Google Calendar attachment sent to the student. On qualification day (firearms example given), the instructor accesses that tier's shooting qualification standard/course of fire, and can record drill times via a "Shooter's Global" shot timer integration or type results in manually. All qualifications are strictly pass/fail, no leniency; any edit to recorded results must leave a verifiable record that an edit was made. After the instructor checks off each qualification item to standard, a Pass button updates the student's profile with the new medal/badge/accomplishment.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Instructor / backend -- Registration, qualification standards, grading</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Broken into S-008 through S-013 (scope items), Q-014 through Q-018 (open questions), and R-003 (risk: qualification record-keeping/compliance). Confirms the earning mechanism behind S-003's rank/medal display and partially answers Q-001 (three pillars = Medical, Firearms, Fitness). Updated Q-002/Q-003 to note the mechanism is known but the actual standards content is still needed from the client.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log role hierarchy, vetting, waivers, locator map, media badges
Capture cofounder Owner role, instructor registration/vetting via a
website, tier upgrade/downgrade-request rule, new-account serial
number issuance, required instructor and universal liability
waivers, zip-code instructor locator map, and quiz-verified media
badges. Add S-014 to S-020, F-001 (future idea), Q-019 to Q-024, and
CAP-009 to CAP-012. Downgrade Q-001 from P0 to P2: the liability
waiver and records-keeping-only business model resolve most of it.
Partially mitigate R-002/R-003 via the waiver, pending enforceability
review. Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). Confirmed user-side flow: branded launch animation -&gt; account login -&gt; individual profile page (photo, current rank, medals/achievements, next-accomplishment guidance) -&gt; tab bar with Home (updates, monthly challenges, community aspect), Chat/Messaging, and a Media tab (medical, fitness, and firearms &amp; building training videos). Three membership tiers gate access: Free (app + profile + Home only), Mid (feature set still being defined by the client), and Premium (all features, including chats, media, challenges, monthly raffles, and additional personalized guidance). The three proficiency pillars are confirmed: Medical, Firearms, and Fitness. Backend/instructor side (new): Approved Instructors share the regular user's profile and access, plus an instructor-only "+" button to pre-register a student for a qualification (category/tier/date), which sends an approval confirmation and a Google Calendar invite to the student. On qualification day, the instructor follows that tier's course-of-fire standard, records results via a shot-timer integration ("Shooter's Global") or manual entry, grades strictly pass/fail with no partial credit, and any edit to results is logged in an audit trail. A Pass automatically updates the student's profile rank/medal. The target audience/business model (who takes this program) is still not stated -- see Q-001.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards, and get an instructor-only "+" button to pre-register students for qualifications (Google Calendar invite sent), access qualification standards on test day, record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos.</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TBD -- not yet explicitly stated by the client.</t>
+          <t>National Proficiency is a records-keeping/tracking company: it documents where people are qualifying (medical, firearms, fitness) and what they currently hold, via vetted Approved Instructors -- it does not set or guarantee the underlying training standards and assumes no liability for outcomes (client's own description). Exact target market/customer segment and monetization beyond the three membership tiers is still not stated -- see Q-001.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Resolve P0 items: business audience/model (Q-001), the actual qualification standards content per category/tier (Q-002, Q-003, S-011), account/auth rules (Q-005), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), and instructor designation process (Q-015).</t>
+          <t>Resolve P0 items: the actual qualification standards content per category/tier (Q-002, Q-003, S-011), account/auth rules including how the unique serial number relates to login (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), and legal review/drafting of both waivers (S-016).</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of navigation structure, monthly-challenge mechanics, Home-vs-Messaging community overlap and tier-gating (Q-004, Q-011), exact Media tab video categories (Q-008), the pre-registration approval workflow (Q-014), Google Calendar integration approach (Q-016), and Shooter's Global integration/partner status (Q-017).</t>
+          <t>Client confirmation of navigation structure, monthly-challenge mechanics, Home-vs-Messaging community overlap and tier-gating (Q-004, Q-011), exact Media tab video categories (Q-008), the pre-registration approval workflow (Q-014), Google Calendar and Shooter's Global integration details (Q-016, Q-017), whether the instructor registration website is a separate build from the app (Q-019), and locator-map search/filter scope (Q-024).</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Login mechanism, profile-page landing screen, tab order, account-required access, the three-tier structure, the three proficiency pillars, strict pass/fail grading, and the edit-audit-trail requirement are decided in direction -- see DECISIONS.md. Mid tier, all pricing, and the full qualification standards content remain undecided.</t>
+          <t>Login mechanism, profile-page landing screen, tab order, account-required access, the three-tier structure, the three proficiency pillars, strict pass/fail grading, the edit-audit-trail requirement, the two-cofounder Owner role, instructor upgrade/no-unilateral-downgrade rule, and both required waivers are decided in direction -- see DECISIONS.md. Mid tier, all pricing, the full qualification standards content, and the actual waiver legal text remain undecided.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>App concept, tier/paywall structure, and instructor/qualification workflow now captured. Still not proposal-ready -- multiple P0 items open, plus legal/compliance risks (R-001 raffle, R-003 qualification record-keeping) that should be reviewed before proposing pricing or timelines. See PROPOSAL_READINESS.md.</t>
+          <t>App concept, tier/paywall structure, instructor/qualification workflow, role hierarchy, and liability model now captured. Still not proposal-ready -- multiple P0 items open, plus legal/compliance risks (R-001 raffle, R-002/R-003 now partially mitigated by the liability waiver but still need enforceability review) that should be resolved before proposing pricing or timelines. See PROPOSAL_READINESS.md.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>What is National Proficiency's target audience and business model? CONFIRMED: the three proficiency pillars are Medical, Firearms, and Fitness, tracked via instructor-administered pass/fail qualification testing. CONFIRMED: completely separate brand/company from Tactical Rabbi, with no crossover of information between the two.</t>
+          <t>What is National Proficiency's target audience and business model? CONFIRMED: three proficiency pillars (Medical, Firearms, Fitness), tracked via vetted-instructor-administered pass/fail testing. CONFIRMED: separate brand from Tactical Rabbi, no crossover. CONFIRMED: business model is records-keeping only -- National Proficiency documents where people qualify and what they hold, and takes no liability for the underlying standards or outcomes (see S-016, R-002, R-003).</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -790,7 +790,7 @@
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Who takes this program (e.g. security professionals, general public, a specific organization's staff), and the business model (training academy selling courses, internal org cert tracking, other) -- still needs to be stated explicitly.</t>
+          <t>Only the specific target market/customer segment (e.g. general public, security professionals, a particular industry) and any monetization beyond the three membership tiers remain unstated -- not proposal-blocking on its own now that the core business model is confirmed.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation in writing.</t>
+          <t>Client confirmation in writing (optional detail).</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>The Media tab hosts firearms training and medical training video content, which may carry liability, age-verification, or regulatory considerations depending on jurisdiction and audience.</t>
+          <t>The Media tab hosts firearms training and medical training video content, which may carry liability, age-verification, or regulatory considerations depending on jurisdiction and audience. PARTIALLY MITIGATED: client confirmed every user signs a liability waiver stating National Proficiency is a records-keeping company only and bears no responsibility for shooting/medical/fitness outcomes (S-016) -- but a waiver's enforceability still needs legal confirmation, especially for firearms/medical content and any age-restricted material.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1532,7 +1532,7 @@
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Legal/compliance review of content liability and any age/identity verification needed before granting Media tab access.</t>
+          <t>Legal/compliance review of content liability, the waiver's actual enforceability in relevant jurisdictions, and any age/identity verification needed before granting Media tab access.</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Account required for all app access -- no guest/anonymous use. New users create an account and select a membership tier; existing users log in with username/password.</t>
+          <t>Account required for all app access -- no guest/anonymous use. New users create an account and select a membership tier; existing users log in. New users provide basic info and are then issued a unique serial number/code used to access their account (S-019).</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1638,7 +1638,7 @@
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Account provisioning method, password-reset flow, session/token expiration, MFA, error/lockout handling (Q-005); confirm tier selection happens at sign-up (see S-007).</t>
+          <t>Account provisioning method, password-reset flow, session/token expiration, MFA, error/lockout handling (Q-005); confirm tier selection happens at sign-up (S-007); clarify how the unique serial number (S-019) relates to login -- is it a replacement credential or an additional ID alongside a username/password (Q-022)?</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Qualification records (especially firearms and medical) likely carry legal/compliance requirements around record retention, access control, and edit chain-of-custody -- reinforced by the client's explicit request for an audit trail on edits.</t>
+          <t>Qualification records (especially firearms and medical) likely carry legal/compliance requirements around record retention, access control, and edit chain-of-custody -- reinforced by the client's explicit request for an audit trail on edits. PARTIALLY MITIGATED: client confirmed the business model is explicitly records-keeping only, with a signed user waiver disclaiming responsibility for outcomes (S-016) -- still need legal confirmation this framing holds up, plus the retention/access rules themselves.</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -2221,7 +2221,7 @@
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Legal/compliance review of qualification record-keeping requirements: retention period, who can access records, and whether the audit-trail format meets any applicable regulatory standard. Related to R-001, R-002.</t>
+          <t>Legal/compliance review of qualification record-keeping requirements: retention period, who can access records (cofounders have full access per S-014 -- confirm that's the intended access model), and whether the audit-trail format meets any applicable regulatory standard. Related to R-001, R-002.</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Qualification grading: instructor checks off each individual qualification criterion (manual notes supported) and grades strictly pass/fail -- no partial/leniency. Any edit to recorded results is logged with an audit trail. On Pass, the student's profile automatically updates with the new medal/badge/accomplishment.</t>
+          <t>Qualification grading: instructor checks off each individual qualification criterion (manual notes supported) and grades strictly pass/fail -- no partial/leniency. Any edit to recorded results is logged with an audit trail. On Pass, the student's profile automatically updates with the new medal/badge/accomplishment (tier upgrade). An instructor cannot lower/remove a student's tier directly -- they can only submit a downgrade request with a required reason (S-018).</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -2550,6 +2550,748 @@
       <c r="K35" s="3" t="inlineStr">
         <is>
           <t>Client confirmation of the pass/fail checklist for one example qualification; QA that an edit after submission creates a visible audit entry; QA that a Pass updates the student's profile rank/medal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="70" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Q-019</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Is the instructor registration website a separate system/build from the mobile app, or a web front-end onto the same backend? Instructors were described as registering "on the website," distinct from how students use the app.</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation of whether a separate web application needs to be scoped and built.</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="70" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Q-020</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Can an instructor register/get approved for more than one specialty category (Firearms, Fitness, Medical), or only one per instructor?</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation of single vs. multi-category instructor certification.</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="70" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Q-021</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Who approves an instructor's tier-downgrade request -- the two cofounders specifically, or another review process? What happens if the request is denied, and is the student notified either way?</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed approval authority and notification behavior for downgrade requests.</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="70" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Q-022</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Is the unique serial number/code issued at account creation a replacement login credential, or an additional ID used alongside a username/password (S-002)? How is it delivered, and can it be recovered or reset if lost?</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Clear definition of the serial number/code's role in authentication, delivery method, and recovery process.</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>User management / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; acceptance criteria for account access using the code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="70" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Q-023</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>What are the specific vetting criteria and process for approving an instructor (e.g. background check, certification proof, references), and who conducts the vetting?</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Documented vetting process and criteria per specialty category.</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>User management / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided vetting checklist or process description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="70" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Q-024</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>For the zip-code-based instructor locator map: what can a user search/filter by (category, specific drill/qualification, distance, availability), and is this feature available to all membership tiers, including Free?</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed search/filter fields and tier availability for the locator map.</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / External integration</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; wireframe review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="70" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>F-001</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media)</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Beyond regular qualification medals, additional leaderboard-style badges people can earn or compete for to rank higher than peers, to build camaraderie.</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Client described this tentatively ("could be") rather than as confirmed scope -- needs confirmation of whether it's intended for v1 or a true future phase, plus leaderboard mechanics and how it relates to the Home tab's community aspect (Q-004, Q-011).</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media) / Reporting</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of scope/timing before any design work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="70" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>S-014</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Cofounder / Owner role: the two highest-level users (the app's cofounders) have access to all instructor and student files/records and can edit any individual part they see fit.</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>How this maps to system permissions (a distinct "Owner" role vs. broader "Admin"), whether cofounder edits are also logged in an audit trail (consistent with S-013's requirement), and whether cofounders are the approval authority for instructor downgrade requests (Q-021).</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the permission model; QA that only the two designated cofounder accounts have full-record edit access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="70" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>S-015</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Instructor registration &amp; vetting: prospective instructors register on a website, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor.</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Whether the registration website is a separate build from the app (Q-019), the specific vetting criteria/process and who conducts it (Q-023), and whether multi-category certification is allowed (Q-020).</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / User management / Public form</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided vetting checklist; QA of the full registration-to-approval flow for one test instructor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="70" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>S-016</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Two required waivers: (1) instructors sign a waiver agreeing to follow National Proficiency's standards; (2) every user signs a liability waiver acknowledging National Proficiency is solely a records-keeping company, takes no responsibility for shooting/medical/fitness qualification standards or outcomes, and that all liability -- including compliance with local, state, and federal law -- rests with the individual.</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Actual waiver legal text (needs to come from the client's legal counsel), e-signature mechanism and storage, versioning if waiver text changes, and confirmation that waiver acceptance gates account/instructor activation. Directly relates to and partially mitigates R-002, R-003 -- but enforceability still needs a legal review.</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Sign-off from client's legal counsel on waiver text; QA that an account/instructor cannot be activated without a recorded signature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="70" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>S-017</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Instructor locator map: a person can search by zip code to find the nearest approved instructors for the specific drills/qualifications they need.</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Search/filter scope (category, specific drill, distance, availability) and tier availability -- see Q-024. Needs a mapping API integration.</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / External integration</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of search/filter fields; QA of search results against a set of test instructor locations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="70" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>S-018</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Tier upgrade / downgrade-request workflow: an instructor can upgrade a student's tier directly upon completing a qualification (via the S-013 Pass flow), but cannot lower or remove a tier directly -- they can only submit a downgrade request, providing a required reason.</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Who approves a downgrade request and what happens if it's denied (Q-021); whether the student is notified when a request is filed and/or resolved; whether supporting evidence beyond a text reason is required.</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the approval workflow; QA that an instructor account cannot directly lower a tier, only submit a request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="70" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>S-019</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>New account creation: an unregistered person creates an account with basic information, after which they are issued a unique serial number/code, specific to them, used to access their account.</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Whether this serial number/code replaces or supplements username/password login (S-002), exact "basic information" fields required, delivery method, and recovery process if lost -- see Q-022.</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>User management / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full sign-up field list and how the code is delivered/used; QA of account access using the issued code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="70" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>S-020</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media)</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Video-completion badges: users can earn a digital badge for a specific Media tab video by passing an online quiz/test showing they paid attention to the content (e.g. a "How to Build an AR-15" video with a quiz, earning a badge on their profile).</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Quiz content/format per video, pass threshold, retake policy, and how many videos need this treatment -- builds on the Media tab (S-006).</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media) / Database / records</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Client-provided example quiz for one video; QA that passing the quiz awards the badge on the profile page.</t>
         </is>
       </c>
     </row>
@@ -2718,7 +3460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3169,6 +3911,198 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>CAP-009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Owner-level record access &amp; edit (full instructor and student files)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Two cofounders only</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Owner/admin console (details TBD)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Confirm this is a distinct permission tier from Admin generally, and whether cofounder edits are also audit-logged like instructor edits (S-013).</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-014.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>CAP-010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Instructor registration &amp; vetting</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Prospective instructors (pre-approval)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>External registration website (Q-019) -&gt; choose specialty -&gt; vetting -&gt; waiver -&gt; Approved Instructor status</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Confirm whether this is a separate web build (Q-019), vetting criteria (Q-023), and multi-category eligibility (Q-020).</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-015, S-016.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>CAP-011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Instructor locator map (zip code search)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>All users (tier TBD)</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Location TBD in nav -- search by zip code</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Confirm search/filter scope and tier availability (Q-024).</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-017.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>CAP-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Client portal (Media)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Video-completion badge (watch + quiz)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Premium tier (Media tab access)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Media tab -&gt; watch video -&gt; take quiz -&gt; badge awarded on profile</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Confirm quiz content/format and pass threshold per video (see S-020).</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-020. Distinct from qualification-based medals (S-013).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -3181,7 +4115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3326,6 +4260,33 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="100" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Client described the role hierarchy and account/legal model: two cofounders have full access to edit any instructor or student record. Instructors register on a website, choose a specialty (Firearms/Fitness/Medical), and are individually vetted before being listed as Approved Instructors; a zip-code-based map lets users find nearby instructors for the drills they need. Instructors can upgrade a student's tier on qualification completion but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. New users create an account with basic info and are issued a unique serial number/code to access their account. Instructors sign a waiver to follow National Proficiency's standards; every user signs a liability waiver stating National Proficiency is solely a records-keeping company with no responsibility for shooting/medical/fitness outcomes -- liability and legal compliance rest with the individual. Separately, on the Media tab: users can earn digital badges by watching a specific video and passing an online quiz (e.g. a "How to Build an AR-15" video); the client also mentioned, more tentatively, additional leaderboard-style badges to rank against peers for camaraderie.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Instructor / backend -- Role hierarchy, vetting, waivers, locator map, media badges</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Broken into S-014 through S-020 (scope items), F-001 (future idea -- leaderboard badges, described tentatively), and Q-019 through Q-024 (open questions). This substantially answers Q-001's business-model question (records-keeping only, no liability for outcomes) -- downgraded Q-001 from P0 to P2 since only the specific target market remains unstated. Also partially mitigates R-002/R-003 via the liability waiver, though enforceability still needs legal review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log leaderboard, wearable integration, and standards document
Capture the client's concrete leaderboard details (Fitness/Firearms,
badges/mile/distance metrics), superseding the earlier tentative
F-001. Add S-021 (leaderboard), S-022 (Garmin/Apple Watch/Strava
integration), F-002 (future idea: virtual qualifications via wearable
data), and R-004 (fraud/verification risk for virtual qualifications).
Flag the unreconciled tension between "register on the website" and
"approval could be done on the app" (Q-019). Note the client's
confirmation that a full qualifications/training standards document
exists and will be provided later, resolving the biggest content gap
once received. Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards, and get an instructor-only "+" button to pre-register students for qualifications (Google Calendar invite sent), access qualification standards on test day, record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards, and get an instructor-only "+" button to pre-register students for qualifications (Google Calendar invite sent), access qualification standards on test day, record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. New: a Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.), fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Resolve P0 items: the actual qualification standards content per category/tier (Q-002, Q-003, S-011), account/auth rules including how the unique serial number relates to login (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), and legal review/drafting of both waivers (S-016).</t>
+          <t>Receive the client's qualifications/training standards document (Q-002, Q-003, S-011) once available. In parallel, resolve P0 items: account/auth rules including the serial number vs. login question (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), whether instructor registration/vetting is web or in-app (Q-019), and legal review/drafting of both waivers (S-016).</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of navigation structure, monthly-challenge mechanics, Home-vs-Messaging community overlap and tier-gating (Q-004, Q-011), exact Media tab video categories (Q-008), the pre-registration approval workflow (Q-014), Google Calendar and Shooter's Global integration details (Q-016, Q-017), whether the instructor registration website is a separate build from the app (Q-019), and locator-map search/filter scope (Q-024).</t>
+          <t>Client confirmation of navigation structure, monthly-challenge mechanics, Home-vs-Messaging community overlap and tier-gating (Q-004, Q-011), exact Media tab video categories (Q-008), the pre-registration approval workflow (Q-014), Google Calendar and Shooter's Global integration details (Q-016, Q-017), leaderboard metric list and Medical inclusion (S-021), wearable-platform data points (S-022), and locator-map search/filter scope (Q-024).</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>What are the specific ranks/levels in the progression system, and what are the criteria to advance from one to the next? Mechanism now confirmed: ranks are earned by passing instructor-administered qualifications (S-011, S-013). Still needed: the actual rank/tier list.</t>
+          <t>What are the specific ranks/levels in the progression system, and what are the criteria to advance from one to the next? Mechanism now confirmed: ranks are earned by passing instructor-administered qualifications (S-011, S-013). Client confirmed a full qualifications/training standards document exists and will be provided on a later date.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -843,7 +843,7 @@
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Full rank list and advancement rules per rank -- likely best provided as the actual qualification standards documents (see S-011) rather than described verbally.</t>
+          <t>Full rank list and advancement rules per rank -- client has confirmed the source document exists and is forthcoming (see S-011); this row stays open until it's received and reviewed.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Client-provided rank list; QA against one test account per rank tier.</t>
+          <t>Client-provided rank list (expected via the forthcoming standards document); QA against one test account per rank tier.</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>What are the specific medals/achievements available, and how is each one earned? Mechanism now confirmed: a medal/badge is awarded automatically when an instructor marks a qualification Pass (S-013). Still needed: the actual medal/achievement list per category/tier.</t>
+          <t>What are the specific medals/achievements available, and how is each one earned? Mechanism now confirmed: a medal/badge is awarded automatically when an instructor marks a qualification Pass (S-013). Client confirmed a full qualifications/training standards document exists and will be provided on a later date.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -896,7 +896,7 @@
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Full medal/achievement list and the qualification each one maps to.</t>
+          <t>Full medal/achievement list and the qualification each one maps to -- expected via the forthcoming standards document (see S-011).</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Home tab: updates feed, monthly challenges, a community aspect. Free tier is described as excluding challenges.</t>
+          <t>Home tab: updates feed, monthly challenges, a community aspect, and now also a Fitness/Firearms leaderboard (S-021).</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1744,7 +1744,7 @@
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Source/authorship of updates, monthly-challenge structure and progress tracking (Q-006), how 'community aspect' differs from the Messaging tab (Q-004), and how tier-gating applies within this single tab (Q-011).</t>
+          <t>Source/authorship of updates, monthly-challenge structure and progress tracking (Q-006), how 'community aspect' differs from the Messaging tab (Q-004) and from the new leaderboard (S-021), and how tier-gating applies within this single tab (Q-011).</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Qualification standards library: on the day of testing, the instructor has access to that tier's qualification standard/course of fire to follow while administering the test.</t>
+          <t>Qualification standards library: on the day of testing, the instructor has access to that tier's qualification standard/course of fire to follow while administering the test. Client confirmed a full qualifications/training document covering all standards exists and will be provided later.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2433,7 +2433,7 @@
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>The actual standards/course-of-fire content for every category x tier combination (ties directly to Q-002, Q-003 -- likely needs to come from the client as source documents), format as a structured checklist, and who maintains/updates standards over time.</t>
+          <t>Waiting on the client's full qualifications/training document (confirmed to exist, no date given). Once received: format as a structured checklist per category x tier, and confirm who maintains/updates standards over time.</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Client to provide the qualification standard documents for at least one category/tier as a working example; QA that the correct standard loads for the selected category/tier.</t>
+          <t>Client to provide the full qualifications/training document; QA that the correct standard loads for the selected category/tier once content is built from it.</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Is the instructor registration website a separate system/build from the mobile app, or a web front-end onto the same backend? Instructors were described as registering "on the website," distinct from how students use the app.</t>
+          <t>Is the instructor registration/vetting process a separate website build, or done within the mobile app? Client originally said instructors "register on the website," then later said the approval process "could be done on the app for vetting" -- these two statements haven't been reconciled yet.</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2592,7 +2592,7 @@
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether a separate web application needs to be scoped and built.</t>
+          <t>Confirmation of whether a separate web application needs to be scoped and built, or whether instructor registration and vetting/approval both happen inside the mobile app (which would remove a whole extra build surface).</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -2910,7 +2910,7 @@
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Client described this tentatively ("could be") rather than as confirmed scope -- needs confirmation of whether it's intended for v1 or a true future phase, plus leaderboard mechanics and how it relates to the Home tab's community aspect (Q-004, Q-011).</t>
+          <t>Superseded by S-021 -- client provided concrete leaderboard details (Home tab, Fitness/Firearms, specific metrics) in a later message, elevating this from a tentative future idea to a scoped item.</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/timing before any design work.</t>
+          <t>See S-021.</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Instructor registration &amp; vetting: prospective instructors register on a website, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor.</t>
+          <t>Instructor registration &amp; vetting: prospective instructors register, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor. Client has since said the vetting/approval step could be done within the app itself.</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -3016,7 +3016,7 @@
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Whether the registration website is a separate build from the app (Q-019), the specific vetting criteria/process and who conducts it (Q-023), and whether multi-category certification is allowed (Q-020).</t>
+          <t>Whether registration and vetting are a separate website build or fully in-app (Q-019 -- client's two statements on this haven't been reconciled), the specific vetting criteria/process and who conducts it (Q-023), and whether multi-category certification is allowed (Q-020).</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
@@ -3292,6 +3292,218 @@
       <c r="K49" s="3" t="inlineStr">
         <is>
           <t>Client-provided example quiz for one video; QA that passing the quiz awards the badge on the profile page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="70" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>S-021</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Home tab leaderboard for Fitness and Firearms: ranks users by badges earned, fastest mile, longest distance, and other similar metrics.</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Whether Medical is intentionally excluded from the leaderboard (client mentioned only Fitness and Firearms) or just not yet described; the full list of tracked metrics beyond badge count/fastest mile/longest distance; whether metrics come from wearable integrations (S-022) or instructor-recorded qualification data; opt-out/privacy for appearing on the leaderboard; tie-breaking rules; relationship to the Home tab's community aspect (S-004, Q-004, Q-011). Supersedes F-001, which described this idea tentatively before these details were given.</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Reporting</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of exact metrics and category inclusion; QA that leaderboard rankings update correctly when a test account's stats change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="70" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>S-022</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Wearable/fitness-platform integration: users can connect a Garmin, Apple Watch, or Strava account (their choice) to sync personal fitness/activity data into the app.</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Which specific data points are pulled from each platform, how this feeds the leaderboard (S-021) and profile, OAuth/authentication per platform, fallback for users who don't connect a platform, and data-privacy/consent for syncing health/fitness data.</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>External integration / Client portal</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of exact data points needed per platform; QA of a successful sync from at least one platform populating the leaderboard/profile correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="70" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>F-002</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Future idea (client's own framing -- "could also be used later"): allow certain qualifications to be completed virtually/remotely using wearable-sourced performance data (S-022) tied to specific events, instead of in-person instructor administration.</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Which qualifications (if any) would be eligible for virtual completion, how "specific events" are defined/administered without an instructor present, and anti-fraud/verification safeguards -- see risk R-004. Not proposal-blocking now per the client's own "later date" framing.</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Admin dashboard / External integration</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of scope/timing before any design work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="70" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4103,6 +4315,102 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>CAP-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Home tab leaderboard (Fitness &amp; Firearms)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Logged-in members (tier availability TBD)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Tab bar -&gt; Home -&gt; leaderboard section</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Confirm full metric list, Medical inclusion/exclusion, and data source (S-022) -- see S-021.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-021. Supersedes F-001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="55" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>CAP-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Wearable/fitness-platform connection (Garmin, Apple Watch, Strava)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Logged-in members who opt in</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Profile or settings -&gt; connect account -&gt; platform OAuth</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Confirm data points per platform and consent/privacy handling -- see S-022.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-022. Feeds S-021 leaderboard; may feed future virtual qualifications (F-002).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4115,7 +4423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4287,6 +4595,33 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="100" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Client clarified the instructor approval process could be done within the app itself for vetting (possible tension with the earlier "register on the website" statement -- not yet reconciled). Client also wants: (1) a Home tab leaderboard for Fitness and Firearms -- most badges earned, fastest mile, longest distance, and similar metrics; (2) integration allowing users to connect a Garmin, Apple Watch, or Strava account (their choice) to post/sync personal activity data, which could later support virtual qualifications tied to specific events. Client confirmed a full document with all qualifications and training information exists and will be provided on a later date.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Instructor vetting / Home leaderboard / Wearable integration / Standards document</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Added S-021 (leaderboard, supersedes the more tentative F-001), S-022 (wearable integration), F-002 (future idea: virtual qualifications), and R-004 (risk: virtual-qualification data falsification). Updated Q-019/S-015 to flag the unreconciled website-vs-in-app vetting statements. Updated Q-002/Q-003/S-011 to note the qualifications/training document is confirmed to exist and is forthcoming -- the single biggest content gap now has a committed source, just not yet a date.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log ID verification and ban enforcement requirements
Capture the client's request for third-party ID verification (e.g.
ID.me) during instructor and student registration, confirming age
18+ and firearm eligibility without storing sensitive ID documents.
Add S-023 (ID verification), S-024 (ban enforcement via identity
match), Q-025 to Q-028, CAP-015/CAP-016, and a new P0 risk R-005:
standard ID-verification vendors typically confirm identity/age, not
firearm-purchase eligibility, which usually needs a separate
NICS-style background check. Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards, and get an instructor-only "+" button to pre-register students for qualifications (Google Calendar invite sent), access qualification standards on test day, record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. New: a Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.), fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards, and get an instructor-only "+" button to pre-register students for qualifications (Google Calendar invite sent), access qualification standards on test day, record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Receive the client's qualifications/training standards document (Q-002, Q-003, S-011) once available. In parallel, resolve P0 items: account/auth rules including the serial number vs. login question (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), whether instructor registration/vetting is web or in-app (Q-019), and legal review/drafting of both waivers (S-016).</t>
+          <t>Receive the client's qualifications/training standards document (Q-002, Q-003, S-011) once available. Resolve the ID-verification vendor scope urgently (Q-025, R-005) -- confirm whether the chosen vendor can actually verify firearm eligibility or only identity/age, since this is a real legal-exposure point. In parallel, resolve P0 items: account/auth rules including the serial number vs. login question (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), whether instructor registration/vetting is web or in-app (Q-019), and legal review/drafting of both waivers (S-016).</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Instructor registration &amp; vetting: prospective instructors register, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor. Client has since said the vetting/approval step could be done within the app itself.</t>
+          <t>Instructor registration &amp; vetting: prospective instructors register, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor. Client has since said the vetting/approval step could be done within the app itself. Registration also includes third-party ID verification (S-023).</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -3016,7 +3016,7 @@
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Whether registration and vetting are a separate website build or fully in-app (Q-019 -- client's two statements on this haven't been reconciled), the specific vetting criteria/process and who conducts it (Q-023), and whether multi-category certification is allowed (Q-020).</t>
+          <t>Whether registration and vetting are a separate website build or fully in-app (Q-019 -- client's two statements on this haven't been reconciled), the specific vetting criteria/process and who conducts it (Q-023), whether multi-category certification is allowed (Q-020), and how ID verification (S-023) sequences with vetting.</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>New account creation: an unregistered person creates an account with basic information, after which they are issued a unique serial number/code, specific to them, used to access their account.</t>
+          <t>New account creation: an unregistered person creates an account with basic information, after which they are issued a unique serial number/code, specific to them, used to access their account. Registration also includes third-party ID verification (S-023).</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
       <c r="H48" s="3" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Whether this serial number/code replaces or supplements username/password login (S-002), exact "basic information" fields required, delivery method, and recovery process if lost -- see Q-022.</t>
+          <t>Whether this serial number/code replaces or supplements username/password login (S-002), exact "basic information" fields required, delivery method, recovery process if lost (Q-022), and how this step sequences with ID verification (S-023).</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
@@ -3457,7 +3457,7 @@
     <row r="53" ht="70" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>Q-025</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -3477,12 +3477,12 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>Which specific third-party ID-verification vendor will be used (client mentioned "ID.me" or similar)? Has it been confirmed that this vendor can verify someone is "legally allowed to own a firearm" -- that determination typically requires a NICS-style background check, distinct from standard identity/age verification, which is what services like ID.me normally provide.</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -3493,15 +3493,386 @@
       <c r="H53" s="3" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr">
         <is>
+          <t>Vendor selection and confirmation of exactly what it verifies (identity + age only, vs. actual firearm-purchase eligibility). See related risk R-005.</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; vendor documentation review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="70" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Q-026</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>What is the ban process -- who decides to ban a user (the cofounders, per S-014?), what are grounds for a ban, and is there an appeal process?</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Documented ban criteria, authority, and appeal process, if any.</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="70" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Q-027</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>If ID verification fails, or a person lacks eligible documentation, are they blocked from the app entirely, or only from firearms-related features (with Medical/Fitness still accessible)?</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed behavior for a failed or incomplete verification.</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; acceptance criteria for a failed-verification account state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="70" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Q-028</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Does the per-verification cost charged by the ID-verification vendor affect tier pricing or the overall business model (see Q-010)?</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Waiting on Client</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Confirmation of whether vendor fees are a pricing input.</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Payments / External integration</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; vendor pricing sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="70" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>R-005</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>"Legally allowed to own a firearm" is a specific legal determination that typically requires a NICS-style background check -- standard ID-verification vendors (e.g. ID.me) generally verify identity and age, not firearm-purchase eligibility. Treating an identity-verification pass as confirmation of firearm eligibility could create a false sense of legal compliance and real liability exposure for National Proficiency, distinct from the liability the user waiver (S-016) covers, since this would be National Proficiency's own verification claim.</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Legal/compliance review of what verification is actually achievable and required, and whether the chosen vendor's service (Q-025) covers it or a separate/additional check is needed. Related to R-002, R-003.</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Sign-off from client's legal counsel; written confirmation from the ID-verification vendor of exactly what their product certifies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="70" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems.</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers.</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="70" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="70" customHeight="1">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr">
+      <c r="J60" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K53" s="3" t="inlineStr">
+      <c r="K60" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -3672,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4411,6 +4782,102 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>CAP-015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (age 18+ and firearm eligibility)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>All new registrants -- students and instructors</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Registration flow -&gt; third-party ID verification step -&gt; pass/fail result</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Confirm vendor and exact verification scope (Q-025); confirm no raw ID documents are stored (R-005).</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>CAP-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement / re-registration block</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Cofounders (issue bans); system (auto-detect on new registration)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>A banned identity attempts to re-register -&gt; system matches against verified identity -&gt; blocked or flagged</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Confirm ban criteria, approval authority, and appeal process (Q-026).</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-024.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -4423,7 +4890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4622,6 +5089,33 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Client wants ID verification integrated into instructor and student registration -- via a third-party service (mentioned "ID.me" or similar) to confirm someone is over 18 and legally allowed to own a firearm, explicitly without National Proficiency storing sensitive ID/legal documents on its own systems. This also enables ban enforcement: if a banned person tries to re-register with new information, the system should recognize their previously verified identity and prevent it.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Registration -- ID verification, ban enforcement</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Added S-023 (ID verification) and S-024 (ban enforcement via identity match). Added Q-025 through Q-028 and R-005 (P0 risk: standard ID-verification vendors typically confirm identity/age, not firearm-purchase eligibility, which usually needs a separate NICS-style background check -- flagged so the client doesn't assume more legal coverage than the vendor actually provides). Cross-referenced S-002, S-015, S-019 since this plugs into the existing registration flows for both instructors and students.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Correct registration flow to student-initiated; add content-visibility rules and profile progression visual
Client corrected the qualification registration flow: students now
initiate from their own profile (auto-restricted to their next
eligible tier, with recommended nearby instructors) rather than
instructors typing in student info. Mark S-009 (old flow) as Removed,
superseded by new S-025. Add S-026 (scoped instructor access to
standards per active registration only), S-028 (Pokemon-style profile
progression visual), and Q-029 to Q-031. Update S-011 with new
content-visibility rules: Medical/Fitness standards fully public,
Firearms exact drills confidential with a public per-tier skills
summary. Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards, and get an instructor-only "+" button to pre-register students for qualifications (Google Calendar invite sent), access qualification standards on test day, record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Approved Instructor role: same profile and access to all regular-user features/pages, plus an instructor-only "+" button (center bottom of the app) that opens qualification-administration tools.</t>
+          <t>Approved Instructor role: same profile and access to all regular-user features/pages, plus instructor-only qualification-administration tools. CORRECTED: the original "+" button pre-registration entry point has moved to the student's profile -- see S-025.</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2274,7 +2274,7 @@
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>How instructors are designated/approved, whether certification is per-category, and how the "+" button and instructor tools stay hidden from non-instructor users -- see Q-015.</t>
+          <t>How instructors are designated/approved, whether certification is per-category, and how instructor-only tools stay hidden from non-instructor users -- see Q-015. Registration is now initiated by the student (S-025), not the instructor.</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of instructor designation process; QA that the "+" button appears only for instructor accounts.</t>
+          <t>Client confirmation of instructor designation process; QA that instructor-only tools are hidden from non-instructor accounts.</t>
         </is>
       </c>
     </row>
@@ -2311,12 +2311,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Student pre-registration form (via the "+" button): instructor selects category (Medical / Firearms / Fitness), level/tier, and qualification date, then submits for approval.</t>
+          <t>SUPERSEDED: instructor manually pre-registers a student by typing in their info, category, tier, and date via a "+" button.</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2327,7 +2327,7 @@
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Full field list beyond category/tier/date (e.g. student lookup/ID, location), whether "approval" is a separate review step or an automatic confirmation, and duplicate/reschedule/cancellation handling -- see Q-014.</t>
+          <t>Client corrected this flow: registration is now student-initiated from their own profile, not instructor-initiated. Superseded by S-025 -- kept here, marked Removed, so the correction is traceable rather than silently overwritten.</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of full form fields and approval workflow; QA of a full registration end to end.</t>
+          <t>See S-025.</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Qualification standards library: on the day of testing, the instructor has access to that tier's qualification standard/course of fire to follow while administering the test. Client confirmed a full qualifications/training document covering all standards exists and will be provided later.</t>
+          <t>Qualification standards library: on the day of testing, the instructor has access to that tier's qualification standard/course of fire to follow while administering the test. Client confirmed a full qualifications/training document covering all standards exists and will be provided later. NEW visibility rule per category: Medical and Fitness standards are fully PUBLIC (visible to everyone) since each tops out at a defined ceiling level. Firearms standards are CONFIDENTIAL -- the exact drills are hidden -- but each tier publicly shows the general skills needed to prepare, without revealing the exact test content. An instructor's access to standards content is scoped to what a specific active student registration requires (S-026), not an open browse of every tier.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2433,7 +2433,7 @@
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Waiting on the client's full qualifications/training document (confirmed to exist, no date given). Once received: format as a structured checklist per category x tier, and confirm who maintains/updates standards over time.</t>
+          <t>Waiting on the client's full qualifications/training document (confirmed to exist, no date given). Once received: format as a structured checklist per category x tier; separate the public Medical/Fitness content from the confidential Firearms content plus its public "skills needed" summary per tier; confirm who maintains/updates standards over time.</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Instructor locator map: a person can search by zip code to find the nearest approved instructors for the specific drills/qualifications they need.</t>
+          <t>Instructor locator map: a person can search by zip code to find the nearest approved instructors for the specific drills/qualifications they need. Related to the newer auto-recommendation flow in S-025 -- unclear whether this standalone map still exists separately or is now just how recommended instructors are displayed after registering (see Q-031).</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -3122,7 +3122,7 @@
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Search/filter scope (category, specific drill, distance, availability) and tier availability -- see Q-024. Needs a mapping API integration.</t>
+          <t>Search/filter scope (category, specific drill, distance, availability) and tier availability -- see Q-024. Needs a mapping API integration. Confirm relationship to S-025's automatic instructor recommendation on registration -- Q-031.</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
@@ -3722,7 +3722,7 @@
     <row r="58" ht="70" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>Q-029</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -3742,12 +3742,12 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems.</t>
+          <t>Client described an instructor-visibility boundary tied to the instructor's own achieved level, but the exact wording was unclear (possible transcription issue): is an instructor ever able to view qualification standards above what a specific student's active registration requires -- e.g. for their own reference -- or is their access strictly limited to exactly what that one registration calls for?</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -3758,24 +3758,24 @@
       <c r="H58" s="3" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers.</t>
+          <t>Precise definition of the instructor access-boundary rule beyond "scoped to the active registration" (S-026).</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation in writing to resolve the unclear phrasing.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="70" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>Q-030</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -3785,22 +3785,22 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>For the profile's rank/medal progression visual (S-028): how many future tiers ahead should be visible-but-locked (just the next one, or all remaining), and is this one combined view or a separate view per category (Medical / Firearms / Fitness)?</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -3811,24 +3811,24 @@
       <c r="H59" s="3" t="inlineStr"/>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Confirmed scope of the locked-preview tiers and whether the visual is per-category or combined.</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client confirmation; wireframe review.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="70" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>Q-031</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -3838,22 +3838,22 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>Does the new automatic instructor-recommendation-on-registration (S-025) replace the standalone zip-code instructor locator map (S-017), or do both exist as separate features?</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -3864,15 +3864,333 @@
       <c r="H60" s="3" t="inlineStr"/>
       <c r="I60" s="3" t="inlineStr">
         <is>
+          <t>Confirmation of whether S-017 remains a general browse/search map, in addition to S-025's recommendation step during registration, or whether one supersedes the other.</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="70" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>S-025</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records / External integration</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="70" customHeight="1">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>S-026</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr"/>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="70" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>S-028</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr"/>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="70" customHeight="1">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems.</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr"/>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers.</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="70" customHeight="1">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="70" customHeight="1">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J60" s="3" t="inlineStr">
+      <c r="J66" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr">
+      <c r="K66" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -4043,7 +4361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4406,22 +4724,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Admin dashboard</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Instructor pre-registration ("+" button)</t>
+          <t>Student-initiated qualification registration (CORRECTED -- was instructor-initiated)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Approved Instructors only</t>
+          <t>Students, from their own profile</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Tab bar -&gt; center "+" button -&gt; registration form (category / tier / date) -&gt; submit</t>
+          <t>Profile -&gt; "Register"/"Choose qualification day" -&gt; pick category -&gt; app restricts to next eligible tier -&gt; recommended instructors shown -&gt; submit</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -4436,13 +4754,13 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Confirm approval workflow (Q-014), full form fields, and Google Calendar integration approach (Q-016).</t>
+          <t>Confirm approval workflow (Q-014), full form fields, and Google Calendar integration approach (Q-016). Corrected from an earlier instructor-initiated design -- see S-025, S-009 (Removed).</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Relates to S-008, S-009, S-010.</t>
+          <t>Relates to S-025, S-010. Supersedes the original instructor-"+"-button version of this row's description.</t>
         </is>
       </c>
     </row>
@@ -4875,6 +5193,102 @@
       <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Relates to S-024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>CAP-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Scoped instructor access to qualification standards</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Approved Instructors, limited to actively-registered students</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Instructor opens a student's active registration -&gt; sees only that course's standard, not other tiers</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Confirm exact access-control mechanics and the unclear boundary raised in Q-029.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-026, S-011.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="55" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>CAP-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Profile rank/medal progression visual ("skill tree")</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>All users, viewing their own profile</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Profile page -&gt; progression view</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Confirm how many locked future tiers are shown and per-category vs. combined view (Q-030).</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-028, S-003.</t>
         </is>
       </c>
     </row>
@@ -4890,7 +5304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5116,6 +5530,33 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Client corrected the registration flow: instead of an instructor typing in a student's info and tier, the student now initiates from their own profile ("Register"/"Choose qualification day"), picks a category (Fitness, Medical, or Firearms), and the app -- already knowing their current tier -- only allows registering for the next eligible tier, then recommends nearby instructors. Instructors can only see qualification data for the specific course a student is actively registering for, not browse other tiers freely. Medical and Fitness standards are fully public (each tops out at a ceiling level); Firearms exact drills are hidden, but each tier shows the general skills needed to prepare. On the profile, in addition to photo and current rank, client wants a Pokemon-style progression visual: earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Registration flow correction / Content visibility / Profile progression visual</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Marked S-009 (old instructor-initiated registration) as Removed, superseded by new S-025 (student-initiated registration with auto-eligibility and instructor recommendation). Updated S-008 to remove the "+" button reference. Added S-026 (scoped instructor access to standards) and S-028 (profile progression visual). Updated S-011 and S-017 to reflect the new content-visibility rules and the overlap with the recommendation engine. Added Q-029 (unclear/possibly garbled instructor-visibility phrasing -- flagged rather than guessed), Q-030, Q-031.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log habit-reminder notifications and photo privacy toggle
Add S-029 (Garmin-style customizable daily habit reminders per
pillar: water/steps for Fitness, dry-fire for Firearms, tourniquet
practice for Medical) and S-030 (optional profile photo privacy
toggle, name/code still shown). Add Q-032 to Q-034 and CAP-019/
CAP-020. Flag Q-033 to confirm the privacy toggle is committed scope
given the client's tentative phrasing, rather than assuming it. Sync
all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3334,7 +3334,7 @@
       <c r="H50" s="3" t="inlineStr"/>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Whether Medical is intentionally excluded from the leaderboard (client mentioned only Fitness and Firearms) or just not yet described; the full list of tracked metrics beyond badge count/fastest mile/longest distance; whether metrics come from wearable integrations (S-022) or instructor-recorded qualification data; opt-out/privacy for appearing on the leaderboard; tie-breaking rules; relationship to the Home tab's community aspect (S-004, Q-004, Q-011). Supersedes F-001, which described this idea tentatively before these details were given.</t>
+          <t>Whether Medical is intentionally excluded from the leaderboard (client mentioned only Fitness and Firearms) or just not yet described; the full list of tracked metrics beyond badge count/fastest mile/longest distance; whether metrics come from wearable integrations (S-022) or instructor-recorded qualification data; opt-out/privacy for appearing on the leaderboard (note: profile photo specifically can be hidden per S-030, name/code still shown); tie-breaking rules; relationship to the Home tab's community aspect (S-004, Q-004, Q-011). Supersedes F-001, which described this idea tentatively before these details were given.</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
@@ -3881,7 +3881,7 @@
     <row r="61" ht="70" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>S-025</t>
+          <t>Q-032</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3891,22 +3891,22 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -3917,24 +3917,24 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records / External integration</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="70" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>S-026</t>
+          <t>Q-033</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -3954,12 +3954,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -3970,24 +3970,24 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Admin dashboard</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>S-028</t>
+          <t>Q-034</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -4007,12 +4007,12 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+          <t>Client confirmation; wireframe/surface review.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="70" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>S-029</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4050,17 +4050,17 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems.</t>
+          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -4076,24 +4076,24 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers.</t>
+          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="70" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>S-030</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -4129,24 +4129,24 @@
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Client portal / Security / compliance</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="70" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>S-025</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4156,22 +4156,22 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -4182,15 +4182,280 @@
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records / External integration</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="70" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>S-026</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="70" customHeight="1">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>S-028</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="70" customHeight="1">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems.</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers.</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="70" customHeight="1">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr"/>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="70" customHeight="1">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr"/>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J66" s="3" t="inlineStr">
+      <c r="J71" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K66" s="3" t="inlineStr">
+      <c r="K71" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -4361,7 +4626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5292,6 +5557,102 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="55" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>CAP-019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Customizable habit-reminder notifications</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>All logged-in users</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Settings/preferences -&gt; enable/disable reminder types per pillar</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Confirm full habit list and whether completion is tracked (Q-032).</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-029.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="55" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>CAP-020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Profile photo privacy toggle</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>All logged-in users (opt-in)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Profile/privacy settings -&gt; hide photo toggle</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Confirm scope/priority (Q-033) and full list of affected surfaces (Q-034).</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-030. Client's own phrasing was tentative.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5304,7 +5665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5557,6 +5918,33 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Client wants Garmin-style customizable habit-reminder notifications per pillar: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice), with user-adjustable preferences. Client also suggested (tentatively -- "might be worth integrating") a privacy option letting a user hide their profile photo from other users, while their name and unique code remain visible.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Notifications / Privacy</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Added S-029 (habit-reminder notifications) and S-030 (profile photo privacy toggle), plus Q-032 through Q-034. Cross-referenced S-030 into S-021's leaderboard privacy note. Flagged Q-033 to confirm whether the privacy toggle is committed scope given the client's tentative phrasing, rather than assuming it's confirmed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Flag minor accounts / future children's program as highest-priority risk
Log the client's request for adults to add linked minor (under-18)
accounts, tied to a described future children's program with
deliberately reduced vetting versus the adult program. Add S-031
(minor account mechanism) and F-003 (future children's program), both
explicitly marked do-not-build-yet. Add R-006 as a P0 risk -- the
highest severity logged for this project -- given the combination of
minors, firearms/medical content, and reduced vetting, which runs
counter to how most jurisdictions regulate adults working with
children. Add Q-035 to Q-039 and CAP-021. Recommend legal counsel
review before any design or build work, and exclude this item from
near-term proposal scope/pricing. Sync all companion Markdown files
with a prominent flag on this item.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Receive the client's qualifications/training standards document (Q-002, Q-003, S-011) once available. Resolve the ID-verification vendor scope urgently (Q-025, R-005) -- confirm whether the chosen vendor can actually verify firearm eligibility or only identity/age, since this is a real legal-exposure point. In parallel, resolve P0 items: account/auth rules including the serial number vs. login question (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), whether instructor registration/vetting is web or in-app (Q-019), and legal review/drafting of both waivers (S-016).</t>
+          <t>TOP PRIORITY: get legal counsel review of the minor/children's-program concept (R-006) before any design or build work touches it -- reduced vetting for a program serving children, combined with firearms/medical content, is a serious legal and child-safety exposure. Also receive the client's qualifications/training standards document (Q-002, Q-003, S-011) once available. Resolve the ID-verification vendor scope (Q-025, R-005) -- confirm whether the chosen vendor can actually verify firearm eligibility or only identity/age. In parallel, resolve P0 items: account/auth rules including the serial number vs. login question (Q-005, Q-022), Mid-tier feature list and tier pricing (Q-009, Q-010), the raffle legal/compliance risk (R-001), instructor vetting criteria and downgrade-approval authority (Q-015, Q-021, Q-023), whether instructor registration/vetting is web or in-app (Q-019), and legal review/drafting of both waivers (S-016).</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3881,7 +3881,7 @@
     <row r="61" ht="70" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Q-032</t>
+          <t>Q-035</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3891,17 +3891,17 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
+          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3917,12 +3917,12 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
+          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
@@ -3934,7 +3934,7 @@
     <row r="62" ht="70" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Q-033</t>
+          <t>Q-036</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
+          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -3970,7 +3970,7 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
+          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
@@ -3980,14 +3980,14 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation; legal review once scope is known.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Q-034</t>
+          <t>Q-037</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -3997,17 +3997,17 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
+          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; wireframe/surface review.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="70" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>S-029</t>
+          <t>Q-038</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4050,22 +4050,22 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -4076,24 +4076,24 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>Security / compliance / User management</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="70" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>S-030</t>
+          <t>Q-039</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4103,22 +4103,22 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4129,24 +4129,24 @@
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+          <t>Confirmed access model for minor accounts.</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="70" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>S-025</t>
+          <t>R-006</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4161,17 +4161,17 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -4182,24 +4182,24 @@
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records / External integration</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="70" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>S-026</t>
+          <t>S-031</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -4209,17 +4209,17 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Admin dashboard</t>
+          <t>User management / Security / compliance</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="70" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>S-028</t>
+          <t>F-003</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -4262,22 +4262,22 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -4288,24 +4288,24 @@
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Security / compliance / Client portal</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="70" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>Q-032</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -4315,22 +4315,22 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems.</t>
+          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -4341,24 +4341,24 @@
       <c r="H69" s="3" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers.</t>
+          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>Q-033</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -4378,12 +4378,12 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -4394,24 +4394,24 @@
       <c r="H70" s="3" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="70" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>Q-034</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -4421,22 +4421,22 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -4447,15 +4447,439 @@
       <c r="H71" s="3" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
+          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; wireframe/surface review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="70" customHeight="1">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>S-029</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr"/>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>Notifications / Client portal</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="70" customHeight="1">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>S-030</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="70" customHeight="1">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>S-025</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records / External integration</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="70" customHeight="1">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>S-026</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr"/>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="70" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>S-028</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr"/>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="70" customHeight="1">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr"/>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="70" customHeight="1">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr"/>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="70" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr"/>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J71" s="3" t="inlineStr">
+      <c r="J79" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K71" s="3" t="inlineStr">
+      <c r="K79" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -4626,7 +5050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5653,6 +6077,54 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="55" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>CAP-021</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Minor/dependent account creation (parent-linked)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Adult (parent) accounts, adding a linked minor account</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Adult profile -&gt; "Add a minor" -&gt; minor gets own individual account</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>DO NOT BUILD until the legal review in R-006 is complete. Confirm near-term vs. future-phase scope (Q-035), pillar eligibility for minors (Q-036), and vetting/consent model (Q-037, Q-038).</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-031, F-003. Highest-risk item logged so far -- see R-006.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -5665,7 +6137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5945,6 +6417,33 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="100" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Client wants adult members to be able to add a minor (child under 18) to their account once registered. Client described a future program for children under 18 with their own individual accounts and their own skill-development growth path, deliberately less strictly monitored/vetted than the adult program, with the level of parental oversight largely left to the parent.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Minor accounts / future children's program</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Added S-031 (minor/dependent account creation) and F-003 (future idea: the full children's program). Flagged R-006 as a P0 risk -- the highest-severity item logged so far -- given the combination of minors, a firearms/medical-training platform, and an explicitly REDUCED vetting standard, which runs counter to how most jurisdictions actually regulate adults working with children (typically stricter, not lighter, background-check requirements). Added Q-035 through Q-039 covering scope timing, pillar eligibility for minors, vetting standard, data/consent (COPPA-adjacent), and minor account access. Recommended legal review before any build work on this area -- did not treat the client's description as something to simply schedule for implementation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log store: merch, affiliate links, and deal updates
Add S-032 (merch store), S-033 (affiliate links for recommended
gear), and S-034 (daily/weekly deal updates). Add Q-040 to Q-043
(e-commerce platform, affiliate network, deal sourcing/cadence, tier
availability) and R-007 (routine FTC affiliate-disclosure compliance
flag). Add CAP-022 to CAP-024. Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3881,7 +3881,7 @@
     <row r="61" ht="70" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Q-035</t>
+          <t>Q-040</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3896,12 +3896,12 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
+          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3917,24 +3917,24 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
+          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of platform choice.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="70" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Q-036</t>
+          <t>Q-041</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -3944,17 +3944,17 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
+          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -3970,24 +3970,24 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
+          <t>Confirmed affiliate network(s) to integrate.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; legal review once scope is known.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Q-037</t>
+          <t>Q-042</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -3997,17 +3997,17 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
+          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
+          <t>Deal-sourcing process and update cadence.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="70" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Q-038</t>
+          <t>Q-043</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4050,17 +4050,17 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
+          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -4076,24 +4076,24 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
+          <t>Confirmed tier availability for the store section.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Payments / Client portal</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="70" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Q-039</t>
+          <t>R-007</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4103,22 +4103,22 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
+          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4129,24 +4129,24 @@
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Confirmed access model for minor accounts.</t>
+          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance / External integration</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Sign-off from client's legal counsel on disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="70" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>R-006</t>
+          <t>S-032</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4156,22 +4156,22 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
+          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -4182,24 +4182,24 @@
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
+          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
+          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="70" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>S-031</t>
+          <t>S-033</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -4209,17 +4209,17 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
+          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
+          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>User management / Security / compliance</t>
+          <t>External integration / Payments</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
+          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="70" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>F-003</t>
+          <t>S-034</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -4262,22 +4262,22 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
+          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -4288,24 +4288,24 @@
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
+          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Client portal</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
+          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="70" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Q-032</t>
+          <t>Q-035</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -4315,17 +4315,17 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
+          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -4341,12 +4341,12 @@
       <c r="H69" s="3" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
+          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
@@ -4358,7 +4358,7 @@
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Q-033</t>
+          <t>Q-036</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
+          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -4394,7 +4394,7 @@
       <c r="H70" s="3" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
+          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
@@ -4404,14 +4404,14 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation; legal review once scope is known.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="70" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Q-034</t>
+          <t>Q-037</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -4421,17 +4421,17 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
+          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -4447,24 +4447,24 @@
       <c r="H71" s="3" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; wireframe/surface review.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="70" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>S-029</t>
+          <t>Q-038</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -4474,22 +4474,22 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -4500,24 +4500,24 @@
       <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>Security / compliance / User management</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="70" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>S-030</t>
+          <t>Q-039</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -4527,22 +4527,22 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -4553,24 +4553,24 @@
       <c r="H73" s="3" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+          <t>Confirmed access model for minor accounts.</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="70" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>S-025</t>
+          <t>R-006</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -4585,17 +4585,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -4606,24 +4606,24 @@
       <c r="H74" s="3" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records / External integration</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="70" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>S-026</t>
+          <t>S-031</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -4633,17 +4633,17 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
@@ -4659,24 +4659,24 @@
       <c r="H75" s="3" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Admin dashboard</t>
+          <t>User management / Security / compliance</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="70" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>S-028</t>
+          <t>F-003</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -4686,22 +4686,22 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -4712,24 +4712,24 @@
       <c r="H76" s="3" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Security / compliance / Client portal</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="70" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>Q-032</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -4739,22 +4739,22 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -4765,24 +4765,24 @@
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="70" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>Q-033</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -4802,12 +4802,12 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -4818,24 +4818,24 @@
       <c r="H78" s="3" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="70" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>Q-034</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -4845,22 +4845,22 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -4871,15 +4871,439 @@
       <c r="H79" s="3" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
+          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation; wireframe/surface review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="70" customHeight="1">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>S-029</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr"/>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>Notifications / Client portal</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="70" customHeight="1">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>S-030</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr"/>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Security / compliance</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="70" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>S-025</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr"/>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records / External integration</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="70" customHeight="1">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>S-026</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr"/>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / Admin dashboard</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="70" customHeight="1">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>S-028</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr"/>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="70" customHeight="1">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr"/>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="70" customHeight="1">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr"/>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="70" customHeight="1">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr"/>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J79" s="3" t="inlineStr">
+      <c r="J87" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K79" s="3" t="inlineStr">
+      <c r="K87" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -5050,7 +5474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6080,27 +6504,27 @@
     <row r="22" ht="55" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>CAP-021</t>
+          <t>CAP-022</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Minor/dependent account creation (parent-linked)</t>
+          <t>Merch store (custom branded merchandise)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Adult (parent) accounts, adding a linked minor account</t>
+          <t>All users (tier TBD)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Adult profile -&gt; "Add a minor" -&gt; minor gets own individual account</t>
+          <t>Store section -&gt; browse -&gt; purchase</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -6110,16 +6534,160 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>DO NOT BUILD until the legal review in R-006 is complete. Confirm near-term vs. future-phase scope (Q-035), pillar eligibility for minors (Q-036), and vetting/consent model (Q-037, Q-038).</t>
+          <t>Confirm e-commerce platform (Q-040) and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr"/>
       <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-032.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="55" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CAP-023</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>External integration</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate links / recommended gear</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>All users (tier TBD)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Store section -&gt; recommended products -&gt; affiliate link out</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Confirm affiliate network(s) (Q-041) and required disclosure language (R-007).</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-033.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="55" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>CAP-024</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Client portal</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Daily/weekly deal updates</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>All users (tier TBD)</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Store section -&gt; deals feed</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Confirm sourcing process and cadence (Q-042).</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-034.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="55" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>CAP-021</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Minor/dependent account creation (parent-linked)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Adult (parent) accounts, adding a linked minor account</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Adult profile -&gt; "Add a minor" -&gt; minor gets own individual account</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>DO NOT BUILD until the legal review in R-006 is complete. Confirm near-term vs. future-phase scope (Q-035), pillar eligibility for minors (Q-036), and vetting/consent model (Q-037, Q-038).</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>Relates to S-031, F-003. Highest-risk item logged so far -- see R-006.</t>
         </is>
@@ -6137,7 +6705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6444,6 +7012,33 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Client wants a store section: custom National-Proficiency-branded merch for sale, affiliate links for recommended products/gear, and daily or weekly deal updates.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Store / Merch / Affiliate / Deals</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Added S-032 (merch store), S-033 (affiliate links), S-034 (deal updates), Q-040 through Q-043, R-007 (FTC affiliate/sponsored-content disclosure compliance), and CAP-022 through CAP-024. Lower-severity, routine addition compared to the last two rounds -- no major risk beyond the standard affiliate-disclosure compliance point.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log future-phase media network and additional-pillars direction
Add F-004 (Media tab growing into an entertainment "network" beyond
training content) and F-005 (expansion beyond the three current
pillars into other neutral categories, e.g. vehicle knowledge --
explains the intentionally generic company name). Add Q-044: whether
to architect the category system and media hosting for extensibility
now, given these stated future directions. Update Q-001 and S-006
with the added context. Both F-items logged as future ideas, not
current scope or commitments, consistent with F-002/F-003 handling.
Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates. Future-phase directions (not current scope): the Media tab could grow into a broader entertainment "network" beyond training content (F-004); the company name is intentionally neutral because the three pillars may expand to other categories later, e.g. vehicle knowledge (F-005) -- worth considering whether to architect the category system and media hosting for extensibility now (Q-044).</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -774,7 +774,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>What is National Proficiency's target audience and business model? CONFIRMED: three proficiency pillars (Medical, Firearms, Fitness), tracked via vetted-instructor-administered pass/fail testing. CONFIRMED: separate brand from Tactical Rabbi, no crossover. CONFIRMED: business model is records-keeping only -- National Proficiency documents where people qualify and what they hold, and takes no liability for the underlying standards or outcomes (see S-016, R-002, R-003).</t>
+          <t>What is National Proficiency's target audience and business model? CONFIRMED: three proficiency pillars (Medical, Firearms, Fitness), tracked via vetted-instructor-administered pass/fail testing. CONFIRMED: separate brand from Tactical Rabbi, no crossover. CONFIRMED: business model is records-keeping only -- National Proficiency documents where people qualify and what they hold, and takes no liability for the underlying standards or outcomes (see S-016, R-002, R-003). CONFIRMED: the name "National Proficiency" is intentionally neutral/generic, because the client intends (long-term, F-005) to expand beyond these three pillars into other neutral educational categories (e.g. vehicle knowledge) to help people become more well-rounded.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Media hosting tab (after Home and Chat), accessible only to premium subscribers: hosts medical training videos, fitness training videos, and firearms &amp; building training videos.</t>
+          <t>Media hosting tab (after Home and Chat), accessible only to premium subscribers: hosts medical training videos, fitness training videos, and firearms &amp; building training videos. Client has since said this is intended, long-term, to grow into a broader "network"-style section with shows and entertainment content too (F-004) -- see Q-044 on whether to architect for that now.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1850,7 +1850,7 @@
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Exact video category definitions (Q-008), video hosting/CDN/storage approach, who uploads content (admin only, presumably), streaming vs. download, captioning/accessibility, and any content liability/compliance review (R-002).</t>
+          <t>Exact video category definitions (Q-008), video hosting/CDN/storage approach, who uploads content (admin only, presumably), streaming vs. download, captioning/accessibility, and any content liability/compliance review (R-002). Consider whether the hosting architecture should accommodate the future network/entertainment expansion (F-004) to avoid costly rework later.</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -3881,7 +3881,7 @@
     <row r="61" ht="70" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Q-040</t>
+          <t>Q-044</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3891,17 +3891,17 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal (Media)</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
+          <t>Given the stated future intent to expand beyond the three pillars (e.g. vehicle knowledge, F-005) and to grow Media into a broader entertainment "network" (F-004), should the current build -- category list, tier system, media hosting -- be architected now for extensibility (e.g. a configurable category list, scalable media infrastructure) rather than hardcoded to the three current pillars? This could affect technical approach and cost now even though the new categories/content themselves aren't needed yet.</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3917,24 +3917,24 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
+          <t>Client/technical decision on whether to invest in extensibility now versus building narrowly for the current three pillars and re-architecting later if/when expansion happens.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Payments / External integration</t>
+          <t>Client portal (Media) / Database / records</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of platform choice.</t>
+          <t>Client and technical-lead discussion; document the trade-off either way.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="70" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Q-041</t>
+          <t>F-004</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -3944,22 +3944,22 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Client portal (Media)</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
+          <t>Future idea (client's own framing -- "in the future", "down the line"): expand the Media tab into a broader "network"-style section hosting not just brand-associated educational videos (medical, firearms, fitness -- the current scope, S-006) but also shows and other entertainment content.</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -3970,24 +3970,24 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Confirmed affiliate network(s) to integrate.</t>
+          <t>Not proposal-blocking now per the client's own framing. Would need a content strategy, production/licensing considerations for entertainment content, and likely much larger media hosting/streaming infrastructure than a training-video library -- worth considering during S-006 architecture (see Q-044) even though this content itself is future-phase.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Client portal (Media) / External integration</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of scope/timing before any design or infrastructure work targets this specifically.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Q-042</t>
+          <t>F-005</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -3997,22 +3997,22 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Database / records</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
+          <t>Future idea (client's own framing -- "more for the future"): expand beyond the three current pillars (Medical, Firearms, Fitness) into other neutral educational categories -- client gave "vehicle knowledge" as an example -- to help people become more well-rounded. Client explained the "National Proficiency" name is intentionally neutral/generic to accommodate this.</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Deal-sourcing process and update cadence.</t>
+          <t>No specific new categories are committed yet beyond the one example given. Not proposal-blocking now, but worth flagging for the technical approach: the category/pillar concept currently appears hardcoded to three values across many scope items (S-003, S-009/S-025, S-011, S-021, S-006); building it as a configurable/extensible list now, rather than three hardcoded values, would avoid costly rework if this expansion happens -- see Q-044.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>Database / records / Client portal</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of scope/timing; architectural discussion on category extensibility before the current pillar system is finalized.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="70" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Q-043</t>
+          <t>Q-040</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
+          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -4076,24 +4076,24 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Confirmed tier availability for the store section.</t>
+          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Payments / Client portal</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of platform choice.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="70" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>R-007</t>
+          <t>Q-041</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4108,17 +4108,17 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
+          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4129,24 +4129,24 @@
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
+          <t>Confirmed affiliate network(s) to integrate.</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel on disclosure language.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="70" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>S-032</t>
+          <t>Q-042</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4161,17 +4161,17 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
+          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -4182,24 +4182,24 @@
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
+          <t>Deal-sourcing process and update cadence.</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Payments / External integration</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="70" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>S-033</t>
+          <t>Q-043</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -4214,17 +4214,17 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
+          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
+          <t>Confirmed tier availability for the store section.</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>External integration / Payments</t>
+          <t>Payments / Client portal</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="70" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>S-034</t>
+          <t>R-007</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -4267,17 +4267,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
+          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -4288,24 +4288,24 @@
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
+          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>Security / compliance / External integration</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
+          <t>Sign-off from client's legal counsel on disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="70" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Q-035</t>
+          <t>S-032</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -4315,22 +4315,22 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
+          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -4341,24 +4341,24 @@
       <c r="H69" s="3" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
+          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Q-036</t>
+          <t>S-033</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4368,22 +4368,22 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
+          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -4394,24 +4394,24 @@
       <c r="H70" s="3" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
+          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration / Payments</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; legal review once scope is known.</t>
+          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="70" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Q-037</t>
+          <t>S-034</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -4421,22 +4421,22 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
+          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -4447,24 +4447,24 @@
       <c r="H71" s="3" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
+          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="70" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Q-038</t>
+          <t>Q-035</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -4474,17 +4474,17 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
+          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -4500,24 +4500,24 @@
       <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
+          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="70" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Q-039</t>
+          <t>Q-036</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -4527,17 +4527,17 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
+          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -4553,24 +4553,24 @@
       <c r="H73" s="3" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Confirmed access model for minor accounts.</t>
+          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation; legal review once scope is known.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="70" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>R-006</t>
+          <t>Q-037</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -4590,12 +4590,12 @@
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
+          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -4606,7 +4606,7 @@
       <c r="H74" s="3" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
+          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
@@ -4616,14 +4616,14 @@
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="70" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>S-031</t>
+          <t>Q-038</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -4633,22 +4633,22 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
+          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -4659,24 +4659,24 @@
       <c r="H75" s="3" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
+          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>User management / Security / compliance</t>
+          <t>Security / compliance / User management</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="70" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>F-003</t>
+          <t>Q-039</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -4686,22 +4686,22 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
+          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -4712,24 +4712,24 @@
       <c r="H76" s="3" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
+          <t>Confirmed access model for minor accounts.</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Client portal</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="70" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Q-032</t>
+          <t>R-006</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -4739,22 +4739,22 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
+          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -4765,24 +4765,24 @@
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
+          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="70" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Q-033</t>
+          <t>S-031</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -4792,22 +4792,22 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
+          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -4818,24 +4818,24 @@
       <c r="H78" s="3" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
+          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management / Security / compliance</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="70" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Q-034</t>
+          <t>F-003</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -4845,22 +4845,22 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
+          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -4871,24 +4871,24 @@
       <c r="H79" s="3" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance / Client portal</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; wireframe/surface review.</t>
+          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="70" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>S-029</t>
+          <t>Q-032</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -4908,12 +4908,12 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -4924,7 +4924,7 @@
       <c r="H80" s="3" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
@@ -4934,14 +4934,14 @@
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="70" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>S-030</t>
+          <t>Q-033</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -4977,24 +4977,24 @@
       <c r="H81" s="3" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Security / compliance</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="70" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>S-025</t>
+          <t>Q-034</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -5014,12 +5014,12 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -5030,24 +5030,24 @@
       <c r="H82" s="3" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records / External integration</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+          <t>Client confirmation; wireframe/surface review.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="70" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>S-026</t>
+          <t>S-029</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5057,17 +5057,17 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
@@ -5083,24 +5083,24 @@
       <c r="H83" s="3" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Admin dashboard</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="70" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>S-028</t>
+          <t>S-030</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -5110,17 +5110,17 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -5136,24 +5136,24 @@
       <c r="H84" s="3" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Client portal / Security / compliance</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="70" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>S-025</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -5168,12 +5168,12 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
@@ -5189,24 +5189,24 @@
       <c r="H85" s="3" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Client portal / Database / records / External integration</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="70" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>S-026</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -5242,24 +5242,24 @@
       <c r="H86" s="3" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Security / compliance / Admin dashboard</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="70" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>S-028</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -5269,22 +5269,22 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -5295,15 +5295,174 @@
       <c r="H87" s="3" t="inlineStr"/>
       <c r="I87" s="3" t="inlineStr">
         <is>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="70" customHeight="1">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr"/>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="70" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr"/>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="70" customHeight="1">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr"/>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J87" s="3" t="inlineStr">
+      <c r="J90" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K87" s="3" t="inlineStr">
+      <c r="K90" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -6705,7 +6864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7039,6 +7198,33 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="100" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Client described two future (not current-scope) directions: (1) the Media tab growing into a broader "network"-style section with shows/entertainment content, beyond today's educational focus (medical, firearms, fitness); (2) the company name "National Proficiency" is intentionally neutral because the client wants to expand beyond the three current pillars into other neutral categories later (e.g. vehicle knowledge), to help people become more well-rounded.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Media network expansion / Additional proficiency categories (future)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Added F-004 (media network/entertainment expansion) and F-005 (additional proficiency categories beyond the three pillars). Both explicitly future-phase per the client's own framing -- not added as current scope. Added Q-044 asking whether the CURRENT build (category list, media hosting) should be architected for extensibility now, given these stated future intentions, since that's a real technical decision even though the expansion itself isn't happening yet. Updated Q-001 and S-006 with the added context.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Correct instructor access to be subscription-gated
Client correction: because the app is subscription-based, Approved
Instructors should not get full regular-user access for free. By
default they get only the instructor module (running/approving
qualifications); full access to messaging, profile/tier progression,
media, etc. requires them to also pay for a subscription like any
other user. Rewrite S-008 in place, update S-007, add Q-045 to Q-047
and CAP-025. Mark the outdated DECISIONS.md entry as superseded
(strikethrough) rather than silently edited, and add the correction
as a new dated entry. Sync all companion Markdown files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates. Future-phase directions (not current scope): the Media tab could grow into a broader entertainment "network" beyond training content (F-004); the company name is intentionally neutral because the three pillars may expand to other categories later, e.g. vehicle knowledge (F-005) -- worth considering whether to architect the category system and media hosting for extensibility now (Q-044).</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates. Future-phase directions (not current scope): the Media tab could grow into a broader entertainment "network" beyond training content (F-004); the company name is intentionally neutral because the three pillars may expand to other categories later, e.g. vehicle knowledge (F-005) -- worth considering whether to architect the category system and media hosting for extensibility now (Q-044). CORRECTED: Approved Instructors do NOT get full regular-user access for free just by being an instructor -- by default they only get the instructor module (running/approving student qualifications). Full access to messaging, their own profile/tier progression, media, and other features requires them to also pay for a subscription (Free/Mid/Premium), same as any other user. This reverses the earlier stated direction for S-008.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Three membership tiers gate feature access. Free: app, profile page, Home page only -- no chats, media, or monthly challenges. Mid: feature set still being defined by the client. Premium: all features, plus monthly raffles tied to challenges, media access, chats, and additional personalized guidance.</t>
+          <t>Three membership tiers gate feature access. Free: app, profile page, Home page only -- no chats, media, or monthly challenges. Mid: feature set still being defined by the client. Premium: all features, plus monthly raffles tied to challenges, media access, chats, and additional personalized guidance. This tier system now also applies to Approved Instructors for anything beyond the instructor module itself -- see S-008 (corrected).</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1903,7 +1903,7 @@
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Full Mid-tier feature list (Q-009), pricing per tier and billing platform (Q-010), upgrade/downgrade flow, and legal review of the raffle mechanic (R-001). This gates the build of nearly every other feature via entitlement/paywall logic.</t>
+          <t>Full Mid-tier feature list (Q-009), pricing per tier and billing platform (Q-010), upgrade/downgrade flow, and legal review of the raffle mechanic (R-001). This gates the build of nearly every other feature via entitlement/paywall logic. Confirm whether instructors pay the same tier pricing as regular users or a distinct instructor subscription price (Q-047).</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Client-provided tier feature matrix and pricing; QA of access boundaries per tier using one test account per tier.</t>
+          <t>Client-provided tier feature matrix and pricing; QA of access boundaries per tier using one test account per tier, including an Approved Instructor account with no paid subscription.</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Approved Instructor role: same profile and access to all regular-user features/pages, plus instructor-only qualification-administration tools. CORRECTED: the original "+" button pre-registration entry point has moved to the student's profile -- see S-025.</t>
+          <t>Approved Instructor role -- CORRECTED (second correction): by default, an Approved Instructor gets access ONLY to the instructor module -- running and approving student qualifications. This reverses the earlier stated direction that instructors get "the same profile and access to all regular-user features/pages." Full access to everything else (messaging, the instructor's own profile/tier progression, media, home feed, leaderboard, etc.) requires the instructor to ALSO pay for a membership subscription (Free/Mid/Premium), same as any other user -- being an Approved Instructor does not itself grant those features for free. The earlier "+" button pre-registration entry point also moved to the student's profile -- see S-025.</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2274,17 +2274,17 @@
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>How instructors are designated/approved, whether certification is per-category, and how instructor-only tools stay hidden from non-instructor users -- see Q-015. Registration is now initiated by the student (S-025), not the instructor.</t>
+          <t>How instructors are designated/approved, whether certification is per-category -- see Q-015. Confirm the exact boundary of "the instructor module" (Q-045): does it include the instructor's own profile/rank tracking, or is that also gated behind a subscription? Confirm what "tier setups" specifically refers to (Q-046). Confirm whether instructors pay the same Free/Mid/Premium pricing as regular users, or a distinct instructor subscription price (Q-047).</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Admin dashboard / User management</t>
+          <t>Admin dashboard / User management / Payments</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of instructor designation process; QA that instructor-only tools are hidden from non-instructor accounts.</t>
+          <t>Client confirmation of the exact instructor-module feature boundary; QA that an unsubscribed Approved Instructor account can run/approve qualifications but is blocked from messaging, tier progression, media, and other member-only features until they subscribe.</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
     <row r="61" ht="70" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Q-044</t>
+          <t>Q-045</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3891,17 +3891,17 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media)</t>
+          <t>Admin dashboard</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Given the stated future intent to expand beyond the three pillars (e.g. vehicle knowledge, F-005) and to grow Media into a broader entertainment "network" (F-004), should the current build -- category list, tier system, media hosting -- be architected now for extensibility (e.g. a configurable category list, scalable media infrastructure) rather than hardcoded to the three current pillars? This could affect technical approach and cost now even though the new categories/content themselves aren't needed yet.</t>
+          <t>What exactly is included in "the instructor module" that an Approved Instructor gets access to without a paid subscription? Does it include the instructor's own profile/rank tracking, or is that also gated behind a subscription like it would be for any other user?</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3917,24 +3917,24 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Client/technical decision on whether to invest in extensibility now versus building narrowly for the current three pillars and re-architecting later if/when expansion happens.</t>
+          <t>Precise feature boundary for the free instructor-only tier of access.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media) / Database / records</t>
+          <t>Admin dashboard</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Client and technical-lead discussion; document the trade-off either way.</t>
+          <t>Client confirmation in writing; acceptance criteria for an unsubscribed instructor account.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="70" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>F-004</t>
+          <t>Q-046</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -3944,22 +3944,22 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media)</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "in the future", "down the line"): expand the Media tab into a broader "network"-style section hosting not just brand-associated educational videos (medical, firearms, fitness -- the current scope, S-006) but also shows and other entertainment content.</t>
+          <t>Client said unsubscribed instructors won't have access to "their tier setups" -- does this mean the instructor's own personal profile/rank progression (S-003), or something else (e.g. admin-configured tier settings)? Wording was ambiguous.</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -3970,24 +3970,24 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Not proposal-blocking now per the client's own framing. Would need a content strategy, production/licensing considerations for entertainment content, and likely much larger media hosting/streaming infrastructure than a training-video library -- worth considering during S-006 architecture (see Q-044) even though this content itself is future-phase.</t>
+          <t>Plain confirmation of what "tier setups" refers to.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media) / External integration</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/timing before any design or infrastructure work targets this specifically.</t>
+          <t>Client confirmation in writing to resolve the ambiguous phrasing.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>F-005</t>
+          <t>Q-047</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -3997,22 +3997,22 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Database / records</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "more for the future"): expand beyond the three current pillars (Medical, Firearms, Fitness) into other neutral educational categories -- client gave "vehicle knowledge" as an example -- to help people become more well-rounded. Client explained the "National Proficiency" name is intentionally neutral/generic to accommodate this.</t>
+          <t>Do Approved Instructors pay the same Free/Mid/Premium subscription pricing as regular users to unlock full app access, or is there a distinct instructor subscription price/tier?</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>No specific new categories are committed yet beyond the one example given. Not proposal-blocking now, but worth flagging for the technical approach: the category/pillar concept currently appears hardcoded to three values across many scope items (S-003, S-009/S-025, S-011, S-021, S-006); building it as a configurable/extensible list now, rather than three hardcoded values, would avoid costly rework if this expansion happens -- see Q-044.</t>
+          <t>Confirmed pricing model for instructors seeking full member access.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>Database / records / Client portal</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/timing; architectural discussion on category extensibility before the current pillar system is finalized.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="70" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Q-040</t>
+          <t>Q-044</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4050,17 +4050,17 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal (Media)</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
+          <t>Given the stated future intent to expand beyond the three pillars (e.g. vehicle knowledge, F-005) and to grow Media into a broader entertainment "network" (F-004), should the current build -- category list, tier system, media hosting -- be architected now for extensibility (e.g. a configurable category list, scalable media infrastructure) rather than hardcoded to the three current pillars? This could affect technical approach and cost now even though the new categories/content themselves aren't needed yet.</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -4076,24 +4076,24 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
+          <t>Client/technical decision on whether to invest in extensibility now versus building narrowly for the current three pillars and re-architecting later if/when expansion happens.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Payments / External integration</t>
+          <t>Client portal (Media) / Database / records</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of platform choice.</t>
+          <t>Client and technical-lead discussion; document the trade-off either way.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="70" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Q-041</t>
+          <t>F-004</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4103,22 +4103,22 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Client portal (Media)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
+          <t>Future idea (client's own framing -- "in the future", "down the line"): expand the Media tab into a broader "network"-style section hosting not just brand-associated educational videos (medical, firearms, fitness -- the current scope, S-006) but also shows and other entertainment content.</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4129,24 +4129,24 @@
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Confirmed affiliate network(s) to integrate.</t>
+          <t>Not proposal-blocking now per the client's own framing. Would need a content strategy, production/licensing considerations for entertainment content, and likely much larger media hosting/streaming infrastructure than a training-video library -- worth considering during S-006 architecture (see Q-044) even though this content itself is future-phase.</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Client portal (Media) / External integration</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of scope/timing before any design or infrastructure work targets this specifically.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="70" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Q-042</t>
+          <t>F-005</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4156,22 +4156,22 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Database / records</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
+          <t>Future idea (client's own framing -- "more for the future"): expand beyond the three current pillars (Medical, Firearms, Fitness) into other neutral educational categories -- client gave "vehicle knowledge" as an example -- to help people become more well-rounded. Client explained the "National Proficiency" name is intentionally neutral/generic to accommodate this.</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -4182,24 +4182,24 @@
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Deal-sourcing process and update cadence.</t>
+          <t>No specific new categories are committed yet beyond the one example given. Not proposal-blocking now, but worth flagging for the technical approach: the category/pillar concept currently appears hardcoded to three values across many scope items (S-003, S-009/S-025, S-011, S-021, S-006); building it as a configurable/extensible list now, rather than three hardcoded values, would avoid costly rework if this expansion happens -- see Q-044.</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>Database / records / Client portal</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of scope/timing; architectural discussion on category extensibility before the current pillar system is finalized.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="70" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Q-043</t>
+          <t>Q-040</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
+          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Confirmed tier availability for the store section.</t>
+          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>Payments / Client portal</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of platform choice.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="70" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>R-007</t>
+          <t>Q-041</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -4267,17 +4267,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
+          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -4288,24 +4288,24 @@
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
+          <t>Confirmed affiliate network(s) to integrate.</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel on disclosure language.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="70" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>S-032</t>
+          <t>Q-042</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -4320,17 +4320,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
+          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -4341,24 +4341,24 @@
       <c r="H69" s="3" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
+          <t>Deal-sourcing process and update cadence.</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>Payments / External integration</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>S-033</t>
+          <t>Q-043</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4373,17 +4373,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
+          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -4394,24 +4394,24 @@
       <c r="H70" s="3" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
+          <t>Confirmed tier availability for the store section.</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>External integration / Payments</t>
+          <t>Payments / Client portal</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="70" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>S-034</t>
+          <t>R-007</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -4426,17 +4426,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
+          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -4447,24 +4447,24 @@
       <c r="H71" s="3" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
+          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>Security / compliance / External integration</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
+          <t>Sign-off from client's legal counsel on disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="70" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Q-035</t>
+          <t>S-032</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -4474,22 +4474,22 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
+          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -4500,24 +4500,24 @@
       <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
+          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="70" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Q-036</t>
+          <t>S-033</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -4527,22 +4527,22 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
+          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -4553,24 +4553,24 @@
       <c r="H73" s="3" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
+          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>External integration / Payments</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; legal review once scope is known.</t>
+          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="70" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Q-037</t>
+          <t>S-034</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -4580,22 +4580,22 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
+          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -4606,24 +4606,24 @@
       <c r="H74" s="3" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
+          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="70" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Q-038</t>
+          <t>Q-035</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -4633,17 +4633,17 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
+          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
@@ -4659,24 +4659,24 @@
       <c r="H75" s="3" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
+          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="70" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Q-039</t>
+          <t>Q-036</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -4686,17 +4686,17 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
+          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
@@ -4712,24 +4712,24 @@
       <c r="H76" s="3" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>Confirmed access model for minor accounts.</t>
+          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation; legal review once scope is known.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="70" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>R-006</t>
+          <t>Q-037</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -4749,12 +4749,12 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
+          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -4765,7 +4765,7 @@
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
+          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
@@ -4775,14 +4775,14 @@
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="70" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>S-031</t>
+          <t>Q-038</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -4792,22 +4792,22 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
+          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -4818,24 +4818,24 @@
       <c r="H78" s="3" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
+          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>User management / Security / compliance</t>
+          <t>Security / compliance / User management</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="70" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>F-003</t>
+          <t>Q-039</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -4845,22 +4845,22 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
+          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -4871,24 +4871,24 @@
       <c r="H79" s="3" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
+          <t>Confirmed access model for minor accounts.</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Client portal</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="70" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Q-032</t>
+          <t>R-006</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -4898,22 +4898,22 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
+          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -4924,24 +4924,24 @@
       <c r="H80" s="3" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
+          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="70" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Q-033</t>
+          <t>S-031</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -4951,22 +4951,22 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
+          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -4977,24 +4977,24 @@
       <c r="H81" s="3" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
+          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management / Security / compliance</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="70" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Q-034</t>
+          <t>F-003</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -5004,22 +5004,22 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
+          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -5030,24 +5030,24 @@
       <c r="H82" s="3" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance / Client portal</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; wireframe/surface review.</t>
+          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="70" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>S-029</t>
+          <t>Q-032</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -5067,12 +5067,12 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -5083,7 +5083,7 @@
       <c r="H83" s="3" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
@@ -5093,14 +5093,14 @@
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="70" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>S-030</t>
+          <t>Q-033</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -5120,12 +5120,12 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -5136,24 +5136,24 @@
       <c r="H84" s="3" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Security / compliance</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="70" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>S-025</t>
+          <t>Q-034</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -5173,12 +5173,12 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -5189,24 +5189,24 @@
       <c r="H85" s="3" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records / External integration</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+          <t>Client confirmation; wireframe/surface review.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="70" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>S-026</t>
+          <t>S-029</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -5216,17 +5216,17 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -5242,24 +5242,24 @@
       <c r="H86" s="3" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Admin dashboard</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="70" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>S-028</t>
+          <t>S-030</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -5269,17 +5269,17 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -5295,24 +5295,24 @@
       <c r="H87" s="3" t="inlineStr"/>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Client portal / Security / compliance</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="70" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>S-025</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -5327,12 +5327,12 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -5348,24 +5348,24 @@
       <c r="H88" s="3" t="inlineStr"/>
       <c r="I88" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Client portal / Database / records / External integration</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="70" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>S-026</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -5401,24 +5401,24 @@
       <c r="H89" s="3" t="inlineStr"/>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Security / compliance / Admin dashboard</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="70" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>S-028</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -5428,22 +5428,22 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -5454,15 +5454,174 @@
       <c r="H90" s="3" t="inlineStr"/>
       <c r="I90" s="3" t="inlineStr">
         <is>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>Client portal / Database / records</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="70" customHeight="1">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>S-023</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr"/>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / External integration / User management</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="70" customHeight="1">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>S-024</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>Needs Clarification</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr"/>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="70" customHeight="1">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J90" s="3" t="inlineStr">
+      <c r="J93" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K90" s="3" t="inlineStr">
+      <c r="K93" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -5633,7 +5792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6807,27 +6966,27 @@
     <row r="25" ht="55" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>CAP-021</t>
+          <t>CAP-025</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Admin dashboard</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Minor/dependent account creation (parent-linked)</t>
+          <t>Instructor access tiering (instructor module vs. full membership) -- CORRECTED</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Adult (parent) accounts, adding a linked minor account</t>
+          <t>Approved Instructors without a paid subscription: instructor module only. With a paid subscription: full member access too.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Adult profile -&gt; "Add a minor" -&gt; minor gets own individual account</t>
+          <t>Approved Instructor account without a subscription -&gt; can run/approve qualifications only; subscribing (Free/Mid/Premium) unlocks messaging, profile/tier progression, media, home, leaderboard, etc.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -6837,16 +6996,64 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>DO NOT BUILD until the legal review in R-006 is complete. Confirm near-term vs. future-phase scope (Q-035), pillar eligibility for minors (Q-036), and vetting/consent model (Q-037, Q-038).</t>
+          <t>Confirm exact instructor-module boundary (Q-045), meaning of "tier setups" (Q-046), and instructor subscription pricing (Q-047). Reverses the earlier stated direction that instructors get full regular-user access by default.</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Relates to S-008 (corrected), S-007. Second correction in this project after the S-009 registration-flow correction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>CAP-021</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>User management</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Minor/dependent account creation (parent-linked)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Adult (parent) accounts, adding a linked minor account</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Adult profile -&gt; "Add a minor" -&gt; minor gets own individual account</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not built yet</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Future Phase</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>DO NOT BUILD until the legal review in R-006 is complete. Confirm near-term vs. future-phase scope (Q-035), pillar eligibility for minors (Q-036), and vetting/consent model (Q-037, Q-038).</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>Relates to S-031, F-003. Highest-risk item logged so far -- see R-006.</t>
         </is>
@@ -6864,7 +7071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7225,6 +7432,33 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="100" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Client corrected the instructor access model: because the app is subscription-based, an Approved Instructor should NOT automatically get full regular-user access just by being an instructor. By default they only get the instructor module -- running and approving student qualifications. Full access to everything else (messaging, their own tier setups, and other features) requires the instructor to also pay for a subscription, same as any other user. This reverses the earlier stated direction (S-008, and a DECISIONS.md entry) that instructors share the same profile/access as regular users.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Instructor access model correction (subscription-gated)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Rewrote S-008 in place to reflect the correction (kept as the same ID since it's the same role concept, just corrected -- unlike the S-009 registration-flow correction, which became a new ID since the whole approach changed). Updated S-007 to note instructors are subject to the same tier system for non-instructor features. Added Q-045 (exact instructor-module boundary), Q-046 (unclear meaning of "tier setups"), Q-047 (instructor subscription pricing), and CAP-025. Corrected the earlier DECISIONS.md entry that stated instructors get full regular-user access, rather than leaving it uncorrected.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Log instructor vetting questionnaire details
Capture example fields for the instructor vetting questionnaire:
certifying organization (NRA, USCCA, or similar), average classes
taught per month, and company website, used to confirm an applicant
runs a real, active organization. Update S-015 and Q-023 (partially
answered, full field list still pending) and CAP-010. Add Q-048:
whether claimed certifications are actively verified with the
issuing organization or self-reported. Sync all companion Markdown
files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CzjbNq7urC5QDg9bG1Cvbv
</commit_message>
<xml_diff>
--- a/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
+++ b/national-proficiency-scope-planning/National_Proficiency_Scope_Planning_Worksheet.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates. Future-phase directions (not current scope): the Media tab could grow into a broader entertainment "network" beyond training content (F-004); the company name is intentionally neutral because the three pillars may expand to other categories later, e.g. vehicle knowledge (F-005) -- worth considering whether to architect the category system and media hosting for extensibility now (Q-044). CORRECTED: Approved Instructors do NOT get full regular-user access for free just by being an instructor -- by default they only get the instructor module (running/approving student qualifications). Full access to messaging, their own profile/tier progression, media, and other features requires them to also pay for a subscription (Free/Mid/Premium), same as any other user. This reverses the earlier stated direction for S-008.</t>
+          <t>National Proficiency is a native mobile app (iOS + Android), account-required (no guest access), completely unrelated to Tactical Rabbi (no information crossover). It is a proficiency records-keeping platform across three pillars -- Medical, Firearms, Fitness -- administered by vetted Approved Instructors; National Proficiency itself takes no responsibility for the underlying qualification standards or outcomes (see Business Goal, R-002/R-003). User-side flow: branded launch animation -&gt; account creation (basic info -&gt; issued a unique serial number/code to access the account) or login -&gt; individual profile page (photo, rank, medals, next-accomplishment guidance) -&gt; tab bar with Home, Chat/Messaging, and Media, tier-gated (Free / Mid TBD / Premium). Instructor/backend side: Approved Instructors register and are vetted via a website (choosing a specialty -- Firearms, Fitness, or Medical), sign a waiver to follow National Proficiency's standards. CORRECTED registration flow: the student, not the instructor, now initiates a qualification registration from their own profile (picking category -- Medical/Firearms/Fitness); the app already knows their current tier and only allows registering for the next eligible one, then recommends nearby instructors (Google Calendar invite sent). Instructors access qualification standards on test day -- scoped only to what an active student registration requires, not a free browse of every tier -- record results (Shooter's Global shot timer or manual entry), and grade strictly pass/fail with a mandatory edit-audit-trail. An instructor can upgrade a student's tier on a Pass, but cannot lower/remove a tier directly -- only submit a downgrade request with a required reason. A zip-code-based locator map lets users find nearby instructors. Two cofounders sit above instructors with full access to edit any student or instructor record. Every user signs a liability waiver: National Proficiency is solely a records-keeping company, not responsible for shooting/medical/fitness outcomes -- that liability, and legal compliance, is the individual's own. Media tab also awards quiz-verified badges for watching specific training videos. A Home tab leaderboard for Fitness and Firearms (badges earned, fastest mile, longest distance, etc.) is fed in part by an optional Garmin/Apple Watch/Strava integration users can connect -- which the client also floated as a possible future basis for virtual, remote qualifications. The client also confirmed a full qualifications/training standards document exists and will be provided later, which should resolve the biggest remaining content gap (Q-002, Q-003, S-011) once received. New: registration (both students and instructors) will include third-party ID verification (e.g. ID.me) confirming the person is 18+ and, per the client, "legally allowed to own a firearm" -- without National Proficiency storing sensitive ID/legal documents itself. This also lets the system detect a banned person trying to re-register under new information. New content-visibility rules: Medical and Fitness qualification standards are fully public (each tops out at a ceiling level); Firearms exact drills stay confidential, but each tier publicly shows the general skills needed to prepare. New profile feature: a Pokemon-style progression visual showing earned tiers/medals in full color, the in-progress tier grayed out, and future tiers blacked-out/locked as a preview. New: Garmin-style customizable habit-reminder notifications per pillar (Fitness: water/steps; Firearms: dry-fire practice; Medical: tourniquet practice), and a tentatively-proposed privacy option to hide a profile photo while name/code stay visible. NEW, HIGH-RISK: client wants adults to be able to add a linked minor (under-18) account, part of a described future program for children with their own growth path -- deliberately less strictly vetted than the adult program, with oversight left to parents. This is flagged as the single highest-priority legal/compliance risk logged for this project (R-006), given the combination of minors, firearms/medical content, and reduced vetting -- do not build until legal counsel reviews it. New (routine): a store section combining a custom merch shop, affiliate links for recommended gear, and daily/weekly deal updates. Future-phase directions (not current scope): the Media tab could grow into a broader entertainment "network" beyond training content (F-004); the company name is intentionally neutral because the three pillars may expand to other categories later, e.g. vehicle knowledge (F-005) -- worth considering whether to architect the category system and media hosting for extensibility now (Q-044). CORRECTED: Approved Instructors do NOT get full regular-user access for free just by being an instructor -- by default they only get the instructor module (running/approving student qualifications). Full access to messaging, their own profile/tier progression, media, and other features requires them to also pay for a subscription (Free/Mid/Premium), same as any other user. This reverses the earlier stated direction for S-008. Instructor vetting now includes a questionnaire: certifying organization (e.g. NRA, USCCA, or similar), average classes taught per month, company website, and similar questions to confirm they run a real, active organization.</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>What are the specific vetting criteria and process for approving an instructor (e.g. background check, certification proof, references), and who conducts the vetting?</t>
+          <t>What are the specific vetting criteria and process for approving an instructor, and who conducts the vetting? PARTIALLY ANSWERED: client provided example questionnaire fields -- which organization they're an approved instructor through (e.g. NRA, USCCA, or similar), how many classes they give per month on average, their company website, and "other data like that."</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2804,7 +2804,7 @@
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Documented vetting process and criteria per specialty category.</t>
+          <t>The full, exhaustive list of questionnaire fields (client gave examples, not a complete list), who reviews/scores the answers (cofounders per S-014, or someone else), and pass/fail or scoring criteria for approval. See also Q-048 on whether claimed certifications are actively verified with the issuing organization or just self-reported.</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Client-provided vetting checklist or process description.</t>
+          <t>Client-provided complete vetting questionnaire and review process.</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Instructor registration &amp; vetting: prospective instructors register, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor. Client has since said the vetting/approval step could be done within the app itself. Registration also includes third-party ID verification (S-023).</t>
+          <t>Instructor registration &amp; vetting: prospective instructors register, choose a specialty (Firearms, Fitness, or Medical), and are individually vetted before being listed as an Approved Instructor. Client has since said the vetting/approval step could be done within the app itself. Registration also includes third-party ID verification (S-023) and a vetting QUESTIONNAIRE: which organization they're an approved instructor through (e.g. NRA, USCCA, or similar), how many classes they give per month on average, their company website, and similar questions to confirm they run a real organization suitable to partner with National Proficiency.</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -3016,7 +3016,7 @@
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Whether registration and vetting are a separate website build or fully in-app (Q-019 -- client's two statements on this haven't been reconciled), the specific vetting criteria/process and who conducts it (Q-023), whether multi-category certification is allowed (Q-020), and how ID verification (S-023) sequences with vetting.</t>
+          <t>Whether registration and vetting are a separate website build or fully in-app (Q-019 -- client's two statements on this haven't been reconciled), the full questionnaire field list and review/approval process (Q-023), whether claimed certifications are actively verified with the issuing organization or self-reported (Q-048), whether multi-category certification is allowed (Q-020), and how ID verification (S-023) sequences with vetting.</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Client-provided vetting checklist; QA of the full registration-to-approval flow for one test instructor.</t>
+          <t>Client-provided complete vetting questionnaire; QA of the full registration-to-approval flow for one test instructor.</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
     <row r="61" ht="70" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Q-045</t>
+          <t>Q-048</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3891,17 +3891,17 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Admin dashboard</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>What exactly is included in "the instructor module" that an Approved Instructor gets access to without a paid subscription? Does it include the instructor's own profile/rank tracking, or is that also gated behind a subscription like it would be for any other user?</t>
+          <t>Will a claimed instructor certification (e.g. NRA, USCCA, or similar organization) be actively verified with the issuing organization, or is this self-reported/trust-based on the questionnaire answer alone?</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3917,24 +3917,24 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Precise feature boundary for the free instructor-only tier of access.</t>
+          <t>Confirmed verification approach for claimed certifications -- affects whether an integration/manual-verification workflow is needed versus a simple text field.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Admin dashboard</t>
+          <t>Security / compliance / External integration</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation in writing; acceptance criteria for an unsubscribed instructor account.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="70" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Q-046</t>
+          <t>Q-045</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -3944,17 +3944,17 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Admin dashboard</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Client said unsubscribed instructors won't have access to "their tier setups" -- does this mean the instructor's own personal profile/rank progression (S-003), or something else (e.g. admin-configured tier settings)? Wording was ambiguous.</t>
+          <t>What exactly is included in "the instructor module" that an Approved Instructor gets access to without a paid subscription? Does it include the instructor's own profile/rank tracking, or is that also gated behind a subscription like it would be for any other user?</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -3970,24 +3970,24 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Plain confirmation of what "tier setups" refers to.</t>
+          <t>Precise feature boundary for the free instructor-only tier of access.</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Admin dashboard</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation in writing to resolve the ambiguous phrasing.</t>
+          <t>Client confirmation in writing; acceptance criteria for an unsubscribed instructor account.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="70" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Q-047</t>
+          <t>Q-046</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -4002,12 +4002,12 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Do Approved Instructors pay the same Free/Mid/Premium subscription pricing as regular users to unlock full app access, or is there a distinct instructor subscription price/tier?</t>
+          <t>Client said unsubscribed instructors won't have access to "their tier setups" -- does this mean the instructor's own personal profile/rank progression (S-003), or something else (e.g. admin-configured tier settings)? Wording was ambiguous.</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Confirmed pricing model for instructors seeking full member access.</t>
+          <t>Plain confirmation of what "tier setups" refers to.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation in writing to resolve the ambiguous phrasing.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="70" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Q-044</t>
+          <t>Q-047</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -4050,17 +4050,17 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media)</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Given the stated future intent to expand beyond the three pillars (e.g. vehicle knowledge, F-005) and to grow Media into a broader entertainment "network" (F-004), should the current build -- category list, tier system, media hosting -- be architected now for extensibility (e.g. a configurable category list, scalable media infrastructure) rather than hardcoded to the three current pillars? This could affect technical approach and cost now even though the new categories/content themselves aren't needed yet.</t>
+          <t>Do Approved Instructors pay the same Free/Mid/Premium subscription pricing as regular users to unlock full app access, or is there a distinct instructor subscription price/tier?</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -4076,24 +4076,24 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Client/technical decision on whether to invest in extensibility now versus building narrowly for the current three pillars and re-architecting later if/when expansion happens.</t>
+          <t>Confirmed pricing model for instructors seeking full member access.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media) / Database / records</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Client and technical-lead discussion; document the trade-off either way.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="70" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>F-004</t>
+          <t>Q-044</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -4113,12 +4113,12 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "in the future", "down the line"): expand the Media tab into a broader "network"-style section hosting not just brand-associated educational videos (medical, firearms, fitness -- the current scope, S-006) but also shows and other entertainment content.</t>
+          <t>Given the stated future intent to expand beyond the three pillars (e.g. vehicle knowledge, F-005) and to grow Media into a broader entertainment "network" (F-004), should the current build -- category list, tier system, media hosting -- be architected now for extensibility (e.g. a configurable category list, scalable media infrastructure) rather than hardcoded to the three current pillars? This could affect technical approach and cost now even though the new categories/content themselves aren't needed yet.</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4129,24 +4129,24 @@
       <c r="H65" s="3" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Not proposal-blocking now per the client's own framing. Would need a content strategy, production/licensing considerations for entertainment content, and likely much larger media hosting/streaming infrastructure than a training-video library -- worth considering during S-006 architecture (see Q-044) even though this content itself is future-phase.</t>
+          <t>Client/technical decision on whether to invest in extensibility now versus building narrowly for the current three pillars and re-architecting later if/when expansion happens.</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>Client portal (Media) / External integration</t>
+          <t>Client portal (Media) / Database / records</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/timing before any design or infrastructure work targets this specifically.</t>
+          <t>Client and technical-lead discussion; document the trade-off either way.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="70" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>F-005</t>
+          <t>F-004</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -4161,12 +4161,12 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Database / records</t>
+          <t>Client portal (Media)</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "more for the future"): expand beyond the three current pillars (Medical, Firearms, Fitness) into other neutral educational categories -- client gave "vehicle knowledge" as an example -- to help people become more well-rounded. Client explained the "National Proficiency" name is intentionally neutral/generic to accommodate this.</t>
+          <t>Future idea (client's own framing -- "in the future", "down the line"): expand the Media tab into a broader "network"-style section hosting not just brand-associated educational videos (medical, firearms, fitness -- the current scope, S-006) but also shows and other entertainment content.</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -4182,24 +4182,24 @@
       <c r="H66" s="3" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>No specific new categories are committed yet beyond the one example given. Not proposal-blocking now, but worth flagging for the technical approach: the category/pillar concept currently appears hardcoded to three values across many scope items (S-003, S-009/S-025, S-011, S-021, S-006); building it as a configurable/extensible list now, rather than three hardcoded values, would avoid costly rework if this expansion happens -- see Q-044.</t>
+          <t>Not proposal-blocking now per the client's own framing. Would need a content strategy, production/licensing considerations for entertainment content, and likely much larger media hosting/streaming infrastructure than a training-video library -- worth considering during S-006 architecture (see Q-044) even though this content itself is future-phase.</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Database / records / Client portal</t>
+          <t>Client portal (Media) / External integration</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/timing; architectural discussion on category extensibility before the current pillar system is finalized.</t>
+          <t>Client confirmation of scope/timing before any design or infrastructure work targets this specifically.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="70" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Q-040</t>
+          <t>F-005</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -4209,22 +4209,22 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Database / records</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
+          <t>Future idea (client's own framing -- "more for the future"): expand beyond the three current pillars (Medical, Firearms, Fitness) into other neutral educational categories -- client gave "vehicle knowledge" as an example -- to help people become more well-rounded. Client explained the "National Proficiency" name is intentionally neutral/generic to accommodate this.</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
+          <t>No specific new categories are committed yet beyond the one example given. Not proposal-blocking now, but worth flagging for the technical approach: the category/pillar concept currently appears hardcoded to three values across many scope items (S-003, S-009/S-025, S-011, S-021, S-006); building it as a configurable/extensible list now, rather than three hardcoded values, would avoid costly rework if this expansion happens -- see Q-044.</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>Payments / External integration</t>
+          <t>Database / records / Client portal</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of platform choice.</t>
+          <t>Client confirmation of scope/timing; architectural discussion on category extensibility before the current pillar system is finalized.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="70" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Q-041</t>
+          <t>Q-040</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -4262,17 +4262,17 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
+          <t>Should the merch store be built as a custom checkout (full payment/inventory/shipping build) or integrated with an existing e-commerce platform (e.g. Shopify, Printful for print-on-demand, WooCommerce)? This significantly affects scope and cost.</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
@@ -4288,24 +4288,24 @@
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Confirmed affiliate network(s) to integrate.</t>
+          <t>Platform decision for the merch store, and who handles fulfillment/shipping.</t>
         </is>
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of platform choice.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="70" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Q-042</t>
+          <t>Q-041</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -4320,12 +4320,12 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
+          <t>Which affiliate program(s)/networks should be integrated (e.g. Amazon Associates, direct brand partnerships)?</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -4341,12 +4341,12 @@
       <c r="H69" s="3" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Deal-sourcing process and update cadence.</t>
+          <t>Confirmed affiliate network(s) to integrate.</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
@@ -4358,7 +4358,7 @@
     <row r="70" ht="70" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Q-043</t>
+          <t>Q-042</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4373,12 +4373,12 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
+          <t>Are daily/weekly deals curated manually by the National Proficiency team, or pulled automatically from an affiliate feed? Client said "daily or weekly" -- cadence not yet decided.</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -4394,12 +4394,12 @@
       <c r="H70" s="3" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Confirmed tier availability for the store section.</t>
+          <t>Deal-sourcing process and update cadence.</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>Payments / Client portal</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
@@ -4411,7 +4411,7 @@
     <row r="71" ht="70" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>R-007</t>
+          <t>Q-043</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -4426,17 +4426,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
+          <t>Is the store (merch, affiliate links, deals) available to all membership tiers, or gated -- consistent with how Media/Chat are tier-gated elsewhere in the app?</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -4447,24 +4447,24 @@
       <c r="H71" s="3" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
+          <t>Confirmed tier availability for the store section.</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration</t>
+          <t>Payments / Client portal</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel on disclosure language.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="70" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>S-032</t>
+          <t>R-007</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -4479,17 +4479,17 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
+          <t>Affiliate links and any sponsored/deal content are subject to FTC endorsement/disclosure requirements in the US -- recommended products and deals need clear, compliant disclosure language.</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -4500,24 +4500,24 @@
       <c r="H72" s="3" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
+          <t>Legal/compliance review of required affiliate and sponsored-content disclosure language before the store section is built or launched.</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>Payments / External integration</t>
+          <t>Security / compliance / External integration</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
+          <t>Sign-off from client's legal counsel on disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="70" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>S-033</t>
+          <t>S-032</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -4532,12 +4532,12 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>External integration</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
+          <t>Merch store: an in-app store selling custom National-Proficiency-branded merchandise.</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -4553,24 +4553,24 @@
       <c r="H73" s="3" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
+          <t>E-commerce platform/vendor decision (Q-040), fulfillment/shipping model, payment processing (ties to Q-010), product catalog management, and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>External integration / Payments</t>
+          <t>Payments / External integration</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
+          <t>Client confirmation of platform choice; QA of a full test purchase end to end.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="70" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>S-034</t>
+          <t>S-033</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -4585,12 +4585,12 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>External integration</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
+          <t>Affiliate links: a section recommending third-party products/gear via affiliate links, generating commission revenue for National Proficiency.</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -4606,24 +4606,24 @@
       <c r="H74" s="3" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
+          <t>Which affiliate network(s) (Q-041), how products are curated per category (medical/firearms/fitness gear), required FTC disclosure language (R-007), and who maintains the links.</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Notifications</t>
+          <t>External integration / Payments</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
+          <t>Client confirmation of affiliate network; QA that links route correctly with tracking; legal review of disclosure language.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="70" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Q-035</t>
+          <t>S-034</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -4633,22 +4633,22 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
+          <t>Daily/weekly deal updates: regularly refreshed deal/promotion content shown in the store section.</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -4659,24 +4659,24 @@
       <c r="H75" s="3" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
+          <t>Deal-sourcing process and cadence (Q-042), whether push notifications alert users to new deals (possible tie-in with S-029's notification infrastructure), and tier availability (Q-043).</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Client portal / Notifications</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Client confirmation of sourcing process and cadence; QA that a new deal appears/notifies correctly.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="70" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Q-036</t>
+          <t>Q-035</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -4686,17 +4686,17 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
+          <t>Is the "add a minor" account-creation option itself needed now, as infrastructure, even though the full minor skill-development program is explicitly described as a future initiative? Or should the entire minor-account feature (including the parent's ability to add one) be deferred to that future phase along with the program itself?</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
@@ -4712,24 +4712,24 @@
       <c r="H76" s="3" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
+          <t>Confirmation of whether S-031 is near-term scope or should move to F-003 (future phase) in its entirety.</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; legal review once scope is known.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="70" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Q-037</t>
+          <t>Q-036</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
+          <t>Will the future minor program include Firearms-related training/qualifications for children under 18, or is it limited to Medical and/or Fitness skill development? This has major legal implications given typical restrictions on minors and firearms.</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -4765,7 +4765,7 @@
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
+          <t>Explicit confirmation of which pillars apply to minors -- this materially changes the legal risk profile (see R-006) and whether the program is feasible as described in most jurisdictions.</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
@@ -4775,14 +4775,14 @@
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel.</t>
+          <t>Client confirmation; legal review once scope is known.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="70" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Q-038</t>
+          <t>Q-037</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
+          <t>What does "less strict vetting" mean concretely for instructors or content serving minors? Many jurisdictions actually require ADDITIONAL background-check requirements (not reduced ones) for adults working with children -- has this been considered, or does it need legal review?</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -4818,12 +4818,12 @@
       <c r="H78" s="3" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
+          <t>Legal confirmation of what vetting standard is actually required (and permitted) for a program serving minors, which may be the opposite of what was described. See R-006.</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
@@ -4835,7 +4835,7 @@
     <row r="79" ht="70" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Q-039</t>
+          <t>Q-038</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -4845,17 +4845,17 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
+          <t>What data is collected about a minor for their account, and what parental-consent mechanism will be used? Relevant to COPPA and similar children's-privacy laws, especially if any minor could be under 13.</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -4871,24 +4871,24 @@
       <c r="H79" s="3" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Confirmed access model for minor accounts.</t>
+          <t>Data-minimization plan and parental-consent flow for minor accounts, reviewed against COPPA and any applicable state/international children's-privacy law.</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance / User management</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Sign-off from client's legal counsel.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="70" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>R-006</t>
+          <t>Q-039</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -4898,22 +4898,22 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
+          <t>How does a minor access their own account -- independent login credentials, or fully managed/accessed through the parent's account?</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -4924,24 +4924,24 @@
       <c r="H80" s="3" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
+          <t>Confirmed access model for minor accounts.</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="70" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>S-031</t>
+          <t>R-006</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -4951,22 +4951,22 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
+          <t>A program for minors (under 18) with explicitly less strict monitoring/vetting than the adult program is a substantial legal and child-safety risk, especially given National Proficiency's core pillars include Firearms and Medical training. Concerns include: children's-data-privacy law compliance (e.g. COPPA); laws governing minors and firearms training, which often require MORE supervision, not less; potential platform liability for connecting minors with instructors under a reduced-vetting standard, regardless of leaving oversight "up to parents"; and background-check requirements for adults working with children, which are commonly stricter than for adult-only programs.</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -4977,24 +4977,24 @@
       <c r="H81" s="3" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
+          <t>Urgent legal review before any minor-facing features are scoped or built. This is flagged as a top-priority risk given the combination of minors, firearms/medical content, and an explicitly reduced vetting standard -- recommend resolving Q-036 and Q-037 as part of that review.</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>User management / Security / compliance</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
+          <t>Sign-off from client's legal counsel; do not begin build work on S-031 or F-003 until this review is complete.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="70" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>F-003</t>
+          <t>S-031</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -5004,22 +5004,22 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
+          <t>Minor/dependent account creation: once an adult is registered, they get the option to add a minor (child under 18) to their account. Each minor gets their own individual account with their own progress/program, linked to the parent.</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Future Phase</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -5030,24 +5030,24 @@
       <c r="H82" s="3" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
+          <t>Whether this entry point is near-term scope or should move with the full program to a future phase (Q-035); how much control/visibility the parent has into the minor's account and data (Q-038); minor account access model (Q-039); how this interacts with the 18+ ID-verification gate (S-023). Do not scope for build until the legal review in R-006 is complete.</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Client portal</t>
+          <t>User management / Security / compliance</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
+          <t>Client and legal confirmation of the account-linking model; QA of a parent adding a linked minor account once legal review clears the feature.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="70" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Q-032</t>
+          <t>F-003</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5057,22 +5057,22 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
+          <t>Future idea (client's own framing -- "in the future"): a separate program for children under 18, offering a growth path into different skill sets, deliberately less strictly monitored/vetted than the adult program, with oversight largely left to parents.</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Waiting on Client</t>
+          <t>Future Phase</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -5083,24 +5083,24 @@
       <c r="H83" s="3" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
+          <t>Not proposal-blocking now per the client's own framing, but carries the most significant legal/child-safety risk logged so far (R-006) -- recommend resolving Q-036, Q-037, Q-038 with legal counsel well before any design or build work begins, given the firearms/medical context.</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>Security / compliance / Client portal</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation.</t>
+          <t>Legal sign-off and client confirmation of program scope before this leaves future-phase status.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="70" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Q-033</t>
+          <t>Q-032</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -5115,12 +5115,12 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
+          <t>Is the habit-reminder feature's list of trackable habits fixed to the examples given (water intake/step count for Fitness, dry-fire practice for Firearms, tourniquet practice for Medical), or open to expansion? Should habit completion be logged/tracked (e.g. streaks), or are these just reminder notifications with no verification?</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -5136,12 +5136,12 @@
       <c r="H84" s="3" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
+          <t>Confirmed habit list per category and whether completion tracking/streaks are in scope.</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
@@ -5153,7 +5153,7 @@
     <row r="85" ht="70" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Q-034</t>
+          <t>Q-033</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -5163,17 +5163,17 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
+          <t>Is the profile-photo privacy toggle (S-030) confirmed scope for v1, or a "nice to have" the client is still weighing? Client's own phrasing ("might be worth integrating") was tentative.</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
@@ -5189,24 +5189,24 @@
       <c r="H85" s="3" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
+          <t>Confirmation of whether this is committed scope or an optional future consideration.</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation; wireframe/surface review.</t>
+          <t>Client confirmation.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="70" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>S-029</t>
+          <t>Q-034</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -5221,17 +5221,17 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
+          <t>In which specific places is a user's name, unique code, and/or photo shown to other users -- leaderboard (S-021), locator map results (S-017), messaging (S-005), qualification records seen by an instructor -- so the photo-privacy toggle's scope is well defined?</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Needs Clarification</t>
+          <t>Waiting on Client</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
@@ -5242,24 +5242,24 @@
       <c r="H86" s="3" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
+          <t>Full list of surfaces where identity elements are shown, and which are affected by the privacy toggle.</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Notifications / Client portal</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
+          <t>Client confirmation; wireframe/surface review.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="70" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>S-030</t>
+          <t>S-029</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -5269,17 +5269,17 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
+          <t>Customizable daily habit-reminder notifications per proficiency pillar, similar to Garmin: Fitness (e.g. water intake, step count), Firearms (e.g. dry-fire practice), Medical (e.g. tourniquet practice). Users can adjust which reminders they receive.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -5295,24 +5295,24 @@
       <c r="H87" s="3" t="inlineStr"/>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
+          <t>Full habit list per category and whether it's expandable (Q-032); whether reminders tie into any completion tracking/streak feature or are simple pings; reminder scheduling/frequency configurability; per-habit opt-in/opt-out granularity; possible tie-in with wearable data (S-022) to confirm actual completion (e.g. step count).</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Security / compliance</t>
+          <t>Notifications / Client portal</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
+          <t>Client confirmation of the full habit list and configurability; QA that a test account can enable/disable individual reminder types and receives the correct notification.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="70" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>S-025</t>
+          <t>S-030</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -5322,17 +5322,17 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
+          <t>Profile photo privacy toggle: a user's name and unique code may be shown to other users, but the client wants an option for them to hide their profile photo specifically.</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -5348,24 +5348,24 @@
       <c r="H88" s="3" t="inlineStr"/>
       <c r="I88" s="3" t="inlineStr">
         <is>
-          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
+          <t>Whether this is confirmed scope or still tentative (Q-033 -- client's own phrasing was "might be worth integrating"); the full list of surfaces where identity is shown so the toggle's effect is well defined (Q-034).</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records / External integration</t>
+          <t>Client portal / Security / compliance</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
+          <t>Client confirmation of scope/priority; QA that a test account with the toggle enabled shows no photo to other users anywhere name/code still appear.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="70" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>S-026</t>
+          <t>S-025</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -5380,12 +5380,12 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
+          <t>Student-initiated qualification registration (corrected flow): from their own profile, a student selects "Register"/"Choose qualification day," picks a category (Medical, Firearms, or Fitness), and the app -- already knowing their current tier from their profile -- only lets them register for their next eligible tier (no skipping ahead). Based on category, tier, and location, the student is recommended nearby instructors to choose from. Supersedes the earlier instructor-initiated flow (S-009, now Removed).</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -5401,24 +5401,24 @@
       <c r="H89" s="3" t="inlineStr"/>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
+          <t>Full field list and flow details (date selection, approval step -- Q-014), how the recommendation engine ranks/filters instructors (ties to S-017 locator map -- Q-031), and confirmation this fully replaces instructor-side manual entry.</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / Admin dashboard</t>
+          <t>Client portal / Database / records / External integration</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
+          <t>Client confirmation of the full corrected flow end to end; QA that a test student account can only select their next eligible tier, never a higher one.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="70" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>S-028</t>
+          <t>S-026</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -5428,17 +5428,17 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Client portal</t>
+          <t>Security / compliance</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
+          <t>Scoped instructor access to qualification standards: an instructor cannot browse qualification data for tiers generally (e.g. "scroll through tier ten") -- they can only see the standard content relevant to the specific course a specific student is actively registered for.</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -5454,24 +5454,24 @@
       <c r="H90" s="3" t="inlineStr"/>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
+          <t>Exact access-control implementation (per-registration grant, expiring after the qualification is graded?), and the unclear boundary condition raised in Q-029.</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>Client portal / Database / records</t>
+          <t>Security / compliance / Admin dashboard</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
+          <t>Client confirmation of the access rule; QA that an instructor account cannot view standards content for a tier with no active matching student registration.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="70" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>S-023</t>
+          <t>S-028</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -5481,17 +5481,17 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance</t>
+          <t>Client portal</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
+          <t>Profile rank/medal progression visual ("skill tree"): shows earned tiers/medals in full color, the in-progress tier (medals still needed to advance) grayed out, and future tiers beyond that blacked-out/locked as a preview -- visible but not selectable or viewable in detail.</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -5507,24 +5507,24 @@
       <c r="H91" s="3" t="inlineStr"/>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
+          <t>How many future tiers are shown locked, and whether this is one combined view or per-category (Q-030); ties directly to S-003 and to the confirmed per-tier content-visibility rules in S-011.</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / External integration / User management</t>
+          <t>Client portal / Database / records</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
+          <t>Client confirmation/wireframe review of the visual; QA against test accounts at different progress states (earned / in-progress / locked).</t>
         </is>
       </c>
     </row>
     <row r="92" ht="70" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>S-024</t>
+          <t>S-023</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
+          <t>ID verification during registration (students and instructors): a third-party service (client mentioned "ID.me" or similar) verifies the person is over 18 and, per the client, "legally allowed to own a firearm," without National Proficiency storing sensitive ID/legal documents on its own systems. Now needs to be reconciled with the new minor/dependent account concept (S-031), which is inherently for under-18 users -- see Q-036.</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -5560,24 +5560,24 @@
       <c r="H92" s="3" t="inlineStr"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+          <t>Vendor selection and confirmation of what it actually verifies (Q-025 -- age/identity vs. actual firearm eligibility, which is a distinct legal question, see R-005); what happens on failed verification (Q-027); data-flow confirmation that only a verification result/token is stored, never raw ID documents; consent/privacy disclosures; whether this applies to all tiers; how this 18+ gate interacts with minor accounts (S-031), which are for users under 18 by definition.</t>
         </is>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>Security / compliance / User management</t>
+          <t>Security / compliance / External integration / User management</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+          <t>Client/legal confirmation of vendor and verification scope; QA that a test registration stores no raw ID document data, only a pass/fail verification result.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="70" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>R-004</t>
+          <t>S-024</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -5597,12 +5597,12 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+          <t>Ban enforcement via identity verification: if a user is banned, the system uses their verified identity (from S-023) to detect and prevent them from re-registering under new account information.</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs Clarification</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -5613,15 +5613,68 @@
       <c r="H93" s="3" t="inlineStr"/>
       <c r="I93" s="3" t="inlineStr">
         <is>
+          <t>Ban criteria and approval authority (Q-026); how a match against a banned identity is detected and handled (auto-block vs. flagged for review); whether an appeal process exists; whether this applies to both instructors and students.</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance / User management</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
+        <is>
+          <t>Client confirmation of the ban process; QA that a banned test identity attempting to re-register with different account details is correctly detected and blocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="70" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>R-004</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Client Kickoff Notes</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Security / compliance</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Virtual/remote qualifications sourced from wearable or fitness-tracker data (F-002) could be vulnerable to falsification -- e.g. GPS spoofing, another person wearing the device, or manipulated app data -- since a qualification is an official pass/fail record.</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
           <t>Anti-fraud/verification safeguards to define before F-002 moves past future-phase status (e.g. live verification, cross-checked timestamps/location, or restricting virtual completion to lower-stakes categories only). Tied to F-002; lower urgency than R-001/R-002/R-003 since the underlying feature is explicitly future-phase.</t>
         </is>
       </c>
-      <c r="J93" s="3" t="inlineStr">
+      <c r="J94" s="3" t="inlineStr">
         <is>
           <t>Security / compliance / External integration</t>
         </is>
       </c>
-      <c r="K93" s="3" t="inlineStr">
+      <c r="K94" s="3" t="inlineStr">
         <is>
           <t>Legal/compliance and product review before F-002 is scoped for build.</t>
         </is>
@@ -6304,7 +6357,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Instructor registration &amp; vetting</t>
+          <t>Instructor registration &amp; vetting (with questionnaire)</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -6314,7 +6367,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>External registration website (Q-019) -&gt; choose specialty -&gt; vetting -&gt; waiver -&gt; Approved Instructor status</t>
+          <t>External registration website (Q-019) -&gt; choose specialty -&gt; vetting questionnaire (certifying org e.g. NRA/USCCA, classes per month, company website) -&gt; waiver -&gt; Approved Instructor status</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -6329,7 +6382,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Confirm whether this is a separate web build (Q-019), vetting criteria (Q-023), and multi-category eligibility (Q-020).</t>
+          <t>Confirm whether this is a separate web build (Q-019), full questionnaire field list and review process (Q-023), certification-verification approach (Q-048), and multi-category eligibility (Q-020).</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
@@ -7071,7 +7124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7459,6 +7512,33 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="100" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Client message (chat)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Client described the instructor-vetting questionnaire (part of registration/approval): which organization they're an approved instructor through (e.g. NRA, USCCA, or similar), how many classes they give per month on average, their company website, and similar questions -- to confirm they're an actual credentialed, active, real organization suitable to partner with National Proficiency.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Instructor vetting questionnaire</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Updated S-015 and Q-023 (previously just asking for vetting criteria in the abstract -- now partially answered with concrete example fields, though the full field list is still needed). Added Q-048 (whether claimed certifications are actively verified with the issuing org or self-reported) and updated CAP-010.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>